<commit_message>
Add PDI blank vehicle details fill-up with per-dealer report
For every dealer in PIDUsers, tests/PDI.spec.ts finds WORKSHOP > PDI rows
with a blank field, fills Engine / Battery / Charger from the VIN Details
sheet in Settings > Admin > Modify vehicle details, saves, and re-opens
each chassis to confirm the DMS kept the values. A timeout triggers a
fresh login and one retry; one dealer failing doesn't stop the others.

The run emails a per-dealer summary with an interactive dashboard and the
Excel attached, only when every blank chassis was updated (CC PDI_CC);
a failed run is red and sends no report. tests/PDIDailyReport.spec.ts
combines the day's runs into one report. Both specs are skipped by a
plain `npm test` and run only via the test:pdi / report:pdi-daily
scripts or run-pdi.bat.

Also: 31 PDI test cases in the test case workbook, README section, and
README converted from UTF-16 to UTF-8 so GitHub can render it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Test Cases/DMS_Automation_Test_Cases.xlsx
+++ b/Test Cases/DMS_Automation_Test_Cases.xlsx
@@ -8,19 +8,20 @@
     <sheet sheetId="2" name="Enquiry List" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="GSTR Report" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="MIS Report Check" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Coverage Gaps" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="PDI Vehicle Details" state="visible" r:id="rId8"/>
+    <sheet sheetId="5" name="Coverage Gaps" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="706" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1073" uniqueCount="589">
   <si>
     <t>River DMS - E2E Automation Test Cases</t>
   </si>
   <si>
-    <t>All test cases executed on 25-Sep-2026 against the live DMS (Microsoft Edge and Google Chrome).</t>
+    <t>Enquiry List, GSTR and MIS test cases executed on 25-Sep-2026; PDI Vehicle Details on 28-Sep-2026 — all against the live DMS (Microsoft Edge and Google Chrome). "Not run yet" = handled in code, not yet seen in a live run.</t>
   </si>
   <si>
     <t>Sheet</t>
@@ -72,6 +73,15 @@
   </si>
   <si>
     <t>npm start   (on a server: CI=1 BROWSER_CHANNEL=chromium node run_mis_check.js)</t>
+  </si>
+  <si>
+    <t>PDI Vehicle Details</t>
+  </si>
+  <si>
+    <t>tests/PDI.spec.ts (+ tests/PDIDailyReport.spec.ts)</t>
+  </si>
+  <si>
+    <t>npm run test:pdi   (dry run: npm run test:pdi:dry; daily report: npm run report:pdi-daily)</t>
   </si>
   <si>
     <t/>
@@ -1183,6 +1193,549 @@
     <t>Used for MIS-02 / MIS-21 on 25-Sep</t>
   </si>
   <si>
+    <t>PDI Vehicle Details - tests/PDI.spec.ts</t>
+  </si>
+  <si>
+    <t>For every dealer in PIDUsers: find WORKSHOP &gt; PDI rows with a blank field, fill Engine / Battery / Charger from the VIN Details sheet in SETTINGS &gt; Admin &gt; Modify vehicle details, Save and confirm; per-dealer report emailed (CC) only when the run fully passes, plus a daily combined report.</t>
+  </si>
+  <si>
+    <t>Run: npm run test:pdi   (dry run: npm run test:pdi:dry, daily report: npm run report:pdi-daily)</t>
+  </si>
+  <si>
+    <t>PDI-01</t>
+  </si>
+  <si>
+    <t>No PIDUsers, or a dealer with a missing / placeholder login</t>
+  </si>
+  <si>
+    <t>PIDUsers empty, or a dealer still on &lt;user&gt;/&lt;password&gt;</t>
+  </si>
+  <si>
+    <t>Start the run</t>
+  </si>
+  <si>
+    <t>Stops before any login, naming the dealer(s); nothing is changed</t>
+  </si>
+  <si>
+    <t>Pass (28-Sep-2026)</t>
+  </si>
+  <si>
+    <t>292006 with &lt;user&gt;/&lt;password&gt;: stopped at once (message wording from an earlier build)</t>
+  </si>
+  <si>
+    <t>PDI-02</t>
+  </si>
+  <si>
+    <t>Unknown dealer code in PDI_DEALER</t>
+  </si>
+  <si>
+    <t>PDI_RUN=1</t>
+  </si>
+  <si>
+    <t>PDI_DEALER=999999 npx playwright test tests/PDI.spec.ts</t>
+  </si>
+  <si>
+    <t>PDI_DEALER=999999</t>
+  </si>
+  <si>
+    <t>Stops at once: "PDI_DEALER: dealer 999999 is not in credentials.json."</t>
+  </si>
+  <si>
+    <t>Exact message seen; no login attempted</t>
+  </si>
+  <si>
+    <t>PDI-03</t>
+  </si>
+  <si>
+    <t>Dealer listed twice in PIDUsers</t>
+  </si>
+  <si>
+    <t>332008 entered twice</t>
+  </si>
+  <si>
+    <t>WARN "listed more than once — running it once"; dealer processed once</t>
+  </si>
+  <si>
+    <t>332008 ran once</t>
+  </si>
+  <si>
+    <t>PDI-04</t>
+  </si>
+  <si>
+    <t>VIN Details workbook missing</t>
+  </si>
+  <si>
+    <t>PDI_VIN_FILE=C:\nope\missing.xlsx npx playwright test tests/PDI.spec.ts</t>
+  </si>
+  <si>
+    <t>PDI_VIN_FILE (missing file)</t>
+  </si>
+  <si>
+    <t>Stops at once: "VIN Details workbook not found ... (set PDI_VIN_FILE)"</t>
+  </si>
+  <si>
+    <t>PDI-05</t>
+  </si>
+  <si>
+    <t>Safety</t>
+  </si>
+  <si>
+    <t>PDI specs are not run by a plain npm test / run-tests.bat</t>
+  </si>
+  <si>
+    <t>PDI_RUN not set</t>
+  </si>
+  <si>
+    <t>npx playwright test tests/PDI.spec.ts tests/PDIDailyReport.spec.ts</t>
+  </si>
+  <si>
+    <t>Both specs skipped — no DMS changes, no email</t>
+  </si>
+  <si>
+    <t>"2 skipped"</t>
+  </si>
+  <si>
+    <t>PDI-06</t>
+  </si>
+  <si>
+    <t>Each PIDUsers dealer logs in</t>
+  </si>
+  <si>
+    <t>Real logins in PIDUsers</t>
+  </si>
+  <si>
+    <t>Dealer Code + Tab, User Name, Password, Sign In; log out / clear session before the next dealer</t>
+  </si>
+  <si>
+    <t>PIDUsers (15 dealers)</t>
+  </si>
+  <si>
+    <t>Dashboard verified for every dealer</t>
+  </si>
+  <si>
+    <t>15/15 dealers across the 28-Sep runs</t>
+  </si>
+  <si>
+    <t>PDI-07</t>
+  </si>
+  <si>
+    <t>Run with several dealers</t>
+  </si>
+  <si>
+    <t>That dealer marked failed (screenshot attached); other dealers still run; test red; no report email</t>
+  </si>
+  <si>
+    <t>Not run yet</t>
+  </si>
+  <si>
+    <t>Handled by the per-dealer try/catch; not yet run against the DMS</t>
+  </si>
+  <si>
+    <t>PDI-08</t>
+  </si>
+  <si>
+    <t>Open WORKSHOP &gt; PDI</t>
+  </si>
+  <si>
+    <t>Click WORKSHOP, then PDI (matched by link, as menu names carry an icon)</t>
+  </si>
+  <si>
+    <t>PDI grid (PDIStockCheckingMain.aspx) is shown</t>
+  </si>
+  <si>
+    <t>Worked for all 15 dealers</t>
+  </si>
+  <si>
+    <t>PDI-09</t>
+  </si>
+  <si>
+    <t>PDI grid</t>
+  </si>
+  <si>
+    <t>Rows with a blank field are found</t>
+  </si>
+  <si>
+    <t>PDI grid loaded</t>
+  </si>
+  <si>
+    <t>Read inputs //input[starts-with(@id,"ctl00_cpMain_grdMain_")], group by row, keep rows with any empty field and save their ChassisNo</t>
+  </si>
+  <si>
+    <t>Chassis numbers listed with the blank field names</t>
+  </si>
+  <si>
+    <t>EngineNo was the blank field on every dealer</t>
+  </si>
+  <si>
+    <t>PDI-10</t>
+  </si>
+  <si>
+    <t>PDI grid is empty</t>
+  </si>
+  <si>
+    <t>Dealer with no vehicles waiting for PDI</t>
+  </si>
+  <si>
+    <t>Open PDI</t>
+  </si>
+  <si>
+    <t>271001</t>
+  </si>
+  <si>
+    <t>"PDI grid is empty", "Nothing to update"; Modify page not opened</t>
+  </si>
+  <si>
+    <t>PDI-11</t>
+  </si>
+  <si>
+    <t>No blank rows</t>
+  </si>
+  <si>
+    <t>Every PDI row filled</t>
+  </si>
+  <si>
+    <t>"0 PDI row(s) with blank fields", "Nothing to update"</t>
+  </si>
+  <si>
+    <t>e.g. 292005, 292010, and dealers re-checked after being updated</t>
+  </si>
+  <si>
+    <t>PDI-12</t>
+  </si>
+  <si>
+    <t>Open SETTINGS &gt; Admin &gt; Modify vehicle details</t>
+  </si>
+  <si>
+    <t>Blank rows found</t>
+  </si>
+  <si>
+    <t>SETTINGS &gt; Admin &gt; Modify vehicle details</t>
+  </si>
+  <si>
+    <t>ChangeChassisNo.aspx is shown</t>
+  </si>
+  <si>
+    <t>PDI-13</t>
+  </si>
+  <si>
+    <t>Modify vehicle</t>
+  </si>
+  <si>
+    <t>Show loads the chassis</t>
+  </si>
+  <si>
+    <t>Modify page open</t>
+  </si>
+  <si>
+    <t>Enter chassis in ctl00$cpMain$IdentifierValue, click Show, wait 10 s</t>
+  </si>
+  <si>
+    <t>Chassis from PDI-09</t>
+  </si>
+  <si>
+    <t>Form shows the same ChassisNo</t>
+  </si>
+  <si>
+    <t>PDI-14</t>
+  </si>
+  <si>
+    <t>Show loads a different vehicle / nothing</t>
+  </si>
+  <si>
+    <t>Show a chassis the DMS can't find</t>
+  </si>
+  <si>
+    <t>Skipped: "Show did not load this vehicle"; nothing saved; test red</t>
+  </si>
+  <si>
+    <t>Handled in code; no such chassis met yet</t>
+  </si>
+  <si>
+    <t>PDI-15</t>
+  </si>
+  <si>
+    <t>VIN lookup</t>
+  </si>
+  <si>
+    <t>Fill details from the VIN Details sheet</t>
+  </si>
+  <si>
+    <t>resources/VIN Details (1).xlsx</t>
+  </si>
+  <si>
+    <t>Find chassis in col A; col C -&gt; EngineNo, col B -&gt; BatteryDetails, col D -&gt; VehicleChargerNo; EditChassisReason = "Details updated"</t>
+  </si>
+  <si>
+    <t>VIN Details (1).xlsx (29,814 VINs)</t>
+  </si>
+  <si>
+    <t>All four fields filled with the sheet's values</t>
+  </si>
+  <si>
+    <t>PDI-16</t>
+  </si>
+  <si>
+    <t>Chassis not in the VIN Details sheet</t>
+  </si>
+  <si>
+    <t>Run with a chassis missing from the sheet</t>
+  </si>
+  <si>
+    <t>Skipped and listed as "Not in VIN Details sheet"; test red; no report email</t>
+  </si>
+  <si>
+    <t>Every chassis on 28-Sep was in the sheet; shown correctly in the dashboard preview with sample data</t>
+  </si>
+  <si>
+    <t>PDI-17</t>
+  </si>
+  <si>
+    <t>Save</t>
+  </si>
+  <si>
+    <t>Save and confirm the DMS kept the values</t>
+  </si>
+  <si>
+    <t>Form filled</t>
+  </si>
+  <si>
+    <t>Click Save (ctl00_cpMain_cmdSave), Show again, compare Engine / Battery / Charger</t>
+  </si>
+  <si>
+    <t>Status "Updated"; chassis number logged</t>
+  </si>
+  <si>
+    <t>160 chassis updated across 12 dealers on 28-Sep</t>
+  </si>
+  <si>
+    <t>PDI-18</t>
+  </si>
+  <si>
+    <t>Save clicked but the values were not kept</t>
+  </si>
+  <si>
+    <t>DMS rejects or ignores the change</t>
+  </si>
+  <si>
+    <t>"Save clicked but values not kept"; test red; no report email</t>
+  </si>
+  <si>
+    <t>Handled in code; not seen yet</t>
+  </si>
+  <si>
+    <t>PDI-19</t>
+  </si>
+  <si>
+    <t>Page times out mid-dealer: recover and retry</t>
+  </si>
+  <si>
+    <t>A click / fill times out (session dropped)</t>
+  </si>
+  <si>
+    <t>Log in again if the form is gone; retry that chassis once; continue with the rest</t>
+  </si>
+  <si>
+    <t>Added after 4 timeouts on 372002 (13:38 run). Those 4 were checked in the DMS afterwards: values match the VIN sheet</t>
+  </si>
+  <si>
+    <t>PDI-20</t>
+  </si>
+  <si>
+    <t>Page cannot be recovered</t>
+  </si>
+  <si>
+    <t>Recovery (re-login) also fails</t>
+  </si>
+  <si>
+    <t>Remaining chassis marked "Not attempted"; finished ones kept; next dealer still runs; test red</t>
+  </si>
+  <si>
+    <t>Handled in code</t>
+  </si>
+  <si>
+    <t>PDI-21</t>
+  </si>
+  <si>
+    <t>Dry run</t>
+  </si>
+  <si>
+    <t>Fill the form without saving</t>
+  </si>
+  <si>
+    <t>PDI_DRY_RUN=1</t>
+  </si>
+  <si>
+    <t>npm run test:pdi:dry</t>
+  </si>
+  <si>
+    <t>Form filled for every blank chassis, Save never clicked; report marked DRY RUN</t>
+  </si>
+  <si>
+    <t>D71001: 10 chassis filled, nothing saved</t>
+  </si>
+  <si>
+    <t>PDI-22</t>
+  </si>
+  <si>
+    <t>Results Excel with a Dealers sheet</t>
+  </si>
+  <si>
+    <t>Run ends</t>
+  </si>
+  <si>
+    <t>Output/PDI_BlankChassis_&lt;time&gt;.xlsx: one row per chassis + every dealer checked</t>
+  </si>
+  <si>
+    <t>PDI-23</t>
+  </si>
+  <si>
+    <t>Results Excel is open in Excel (locked)</t>
+  </si>
+  <si>
+    <t>File locked</t>
+  </si>
+  <si>
+    <t>Run ends / daily report written</t>
+  </si>
+  <si>
+    <t>Saved beside it as &lt;name&gt;_&lt;timestamp&gt;.xlsx; run continues</t>
+  </si>
+  <si>
+    <t>Locked PDI_Daily_2026-09-28.xlsx: EBUSY -&gt; saved as _1790610722383.xlsx, report still built</t>
+  </si>
+  <si>
+    <t>PDI-24</t>
+  </si>
+  <si>
+    <t>Report email with dashboard and Excel</t>
+  </si>
+  <si>
+    <t>Passing run ends</t>
+  </si>
+  <si>
+    <t>HTML summary per dealer in the body; PDI_Dashboard.html and the Excel attached</t>
+  </si>
+  <si>
+    <t>Emailed on 28-Sep (before the CC list was added)</t>
+  </si>
+  <si>
+    <t>PDI-25</t>
+  </si>
+  <si>
+    <t>CC list on a passing run</t>
+  </si>
+  <si>
+    <t>PDI_CC in .env</t>
+  </si>
+  <si>
+    <t>Passing real (not dry) run ends</t>
+  </si>
+  <si>
+    <t>Email goes to GMAIL_TO with the PDI_CC people on CC</t>
+  </si>
+  <si>
+    <t>Rule checked with data; the first CC email will be the next passing run</t>
+  </si>
+  <si>
+    <t>PDI-26</t>
+  </si>
+  <si>
+    <t>Failed run sends no report</t>
+  </si>
+  <si>
+    <t>Run with any timeout, missing VIN, values not kept, or failed dealer</t>
+  </si>
+  <si>
+    <t>No PDI report emailed to anyone; test red; dashboard and Excel still saved</t>
+  </si>
+  <si>
+    <t>Rule checked with sample data (1 timeout / failed login / not in VIN sheet -&gt; not sent); not yet seen in a live run</t>
+  </si>
+  <si>
+    <t>PDI-27</t>
+  </si>
+  <si>
+    <t>Dry-run report goes only to GMAIL_TO</t>
+  </si>
+  <si>
+    <t>Dry run ends</t>
+  </si>
+  <si>
+    <t>Email marked DRY RUN, no CC</t>
+  </si>
+  <si>
+    <t>PDI-28</t>
+  </si>
+  <si>
+    <t>Dashboard</t>
+  </si>
+  <si>
+    <t>Interactive dashboard</t>
+  </si>
+  <si>
+    <t>PDI_Dashboard.html</t>
+  </si>
+  <si>
+    <t>Open in a browser; click a dealer bar, outcome chips, search, sort columns, theme toggle, phone width</t>
+  </si>
+  <si>
+    <t>Table filters / sorts correctly; dark mode and phone layout work</t>
+  </si>
+  <si>
+    <t>Sample data: dealer + Error filter -&gt; "2 of 14"; no script errors; no sideways scroll at 390 px</t>
+  </si>
+  <si>
+    <t>PDI-29</t>
+  </si>
+  <si>
+    <t>Daily report</t>
+  </si>
+  <si>
+    <t>Combine the day's runs into one report</t>
+  </si>
+  <si>
+    <t>Result files in Output</t>
+  </si>
+  <si>
+    <t>npm run report:pdi-daily</t>
+  </si>
+  <si>
+    <t>Latest result per chassis; dry runs left out; errors cleared by a later check shown as Updated</t>
+  </si>
+  <si>
+    <t>28-Sep: 5 runs -&gt; 160 chassis, 15 dealers; 372002's 4 timeouts shown as Updated</t>
+  </si>
+  <si>
+    <t>PDI-30</t>
+  </si>
+  <si>
+    <t>No runs on that day</t>
+  </si>
+  <si>
+    <t>PDI_REPORT_DATE=2020-01-01 npm run report:pdi-daily</t>
+  </si>
+  <si>
+    <t>PDI_REPORT_DATE=2020-01-01</t>
+  </si>
+  <si>
+    <t>Stops: "No PDI result files from 2020-01-01"</t>
+  </si>
+  <si>
+    <t>Exact message seen</t>
+  </si>
+  <si>
+    <t>PDI-31</t>
+  </si>
+  <si>
+    <t>Build the report without emailing</t>
+  </si>
+  <si>
+    <t>PDI_SEND_EMAIL=0</t>
+  </si>
+  <si>
+    <t>"report email skipped"; dashboard and Excel still saved</t>
+  </si>
+  <si>
     <t>Item</t>
   </si>
   <si>
@@ -1223,6 +1776,33 @@
   </si>
   <si>
     <t>Add the secrets, then run the workflow manually once</t>
+  </si>
+  <si>
+    <t>tests/PDI.spec.ts — PDI grid size</t>
+  </si>
+  <si>
+    <t>Only the rows the PDI page shows are checked (Top N = 25 by default); blank rows further down are missed</t>
+  </si>
+  <si>
+    <t>Set the Top N box higher before reading the grid if a dealer can have more than 25 vehicles waiting</t>
+  </si>
+  <si>
+    <t>tests/PDI.spec.ts — not yet run live</t>
+  </si>
+  <si>
+    <t>PDI-07, 14, 16, 18, 19, 20, 25, 26, 27 are handled in code but have not happened in a real run yet</t>
+  </si>
+  <si>
+    <t>Mark them Pass the first time each one is seen</t>
+  </si>
+  <si>
+    <t>tests/PDI.spec.ts — fixed 10 s wait after Show</t>
+  </si>
+  <si>
+    <t>Asked for by the process; slow DMS responses beyond 10 s are caught by the ChassisNo check (PDI-14) but not waited for</t>
+  </si>
+  <si>
+    <t>Keep; switch to waiting for the ChassisNo field if it proves flaky</t>
   </si>
 </sst>
 </file>
@@ -1701,7 +2281,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1839,29 +2419,55 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="5">
+        <v>31</v>
+      </c>
+      <c r="D8" s="5">
+        <v>14</v>
+      </c>
+      <c r="E8" s="5">
+        <v>12</v>
+      </c>
+      <c r="F8" s="5">
+        <v>5</v>
+      </c>
+      <c r="G8" s="5">
+        <v>22</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="6">
-        <v>57</v>
-      </c>
-      <c r="D8" s="6">
-        <v>35</v>
-      </c>
-      <c r="E8" s="6">
-        <v>12</v>
-      </c>
-      <c r="F8" s="6">
-        <v>10</v>
-      </c>
-      <c r="G8" s="6">
-        <v>57</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>19</v>
+      <c r="B9" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="6">
+        <v>88</v>
+      </c>
+      <c r="D9" s="6">
+        <v>49</v>
+      </c>
+      <c r="E9" s="6">
+        <v>24</v>
+      </c>
+      <c r="F9" s="6">
+        <v>15</v>
+      </c>
+      <c r="G9" s="6">
+        <v>79</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -1873,9 +2479,10 @@
     <hyperlink ref="A5" r:id="rId1" location="#'Enquiry List'!A1"/>
     <hyperlink ref="A6" r:id="rId2" location="#'GSTR Report'!A1"/>
     <hyperlink ref="A7" r:id="rId3" location="#'MIS Report Check'!A1"/>
+    <hyperlink ref="A8" r:id="rId4" location="#'PDI Vehicle Details'!A1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1898,7 +2505,7 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -1913,7 +2520,7 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1928,7 +2535,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -1943,527 +2550,527 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K5" s="11" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K7" s="11" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="J8" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D9" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K9" s="11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>7</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="J10" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K10" s="11" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D11" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="J11" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K11" s="11" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D12" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="J12" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K12" s="11" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="13" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D13" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="J13" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K13" s="11" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="J14" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D15" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="J15" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D16" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="J16" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K16" s="11" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D17" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="J17" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K17" s="11" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D18" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="J18" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K18" s="11" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -2474,7 +3081,7 @@
     <mergeCell ref="A3:K3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2497,7 +3104,7 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -2512,7 +3119,7 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -2527,7 +3134,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -2542,737 +3149,737 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>6</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K5" s="11" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>6</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K7" s="11" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="J8" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D9" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K9" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>7</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="J10" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K10" s="11" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D11" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="J11" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K11" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="D12" s="14" t="s">
         <v>7</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="J12" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K12" s="11" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="D13" s="14" t="s">
         <v>7</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="J13" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K13" s="11" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="J14" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D15" s="14" t="s">
         <v>7</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="J15" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="D16" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="J16" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K16" s="11" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D17" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="J17" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K17" s="11" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="18" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="D18" s="14" t="s">
         <v>7</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="J18" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K18" s="11" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>6</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="J19" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K19" s="11" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="D20" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="H20" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="J20" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K20" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>6</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="J21" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K21" s="11" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="D22" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="H22" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="J22" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K22" s="11" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="D23" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="J23" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K23" s="11" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="D24" s="15" t="s">
         <v>6</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="H24" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="J24" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K24" s="11" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>
@@ -3283,7 +3890,7 @@
     <mergeCell ref="A3:K3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3306,7 +3913,7 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -3321,7 +3928,7 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -3336,7 +3943,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -3351,842 +3958,2140 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K5" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>6</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K7" s="11" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="J8" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D9" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K9" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>7</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="J10" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K10" s="11" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="D11" s="15" t="s">
         <v>6</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="J11" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K11" s="11" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="D12" s="15" t="s">
         <v>6</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="J12" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K12" s="11" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="D13" s="15" t="s">
         <v>6</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="J13" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K13" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" ht="75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="D14" s="14" t="s">
         <v>7</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="J14" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="D15" s="14" t="s">
         <v>7</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="J15" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="D16" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="J16" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K16" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="D17" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="J17" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K17" s="11" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="18" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="D18" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="J18" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K18" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="D19" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="J19" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K19" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="D20" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="H20" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="J20" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K20" s="11" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="D21" s="14" t="s">
         <v>7</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="J21" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K21" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="D22" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="H22" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="J22" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K22" s="11" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="D23" s="15" t="s">
         <v>6</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="J23" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K23" s="11" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
     </row>
     <row r="24" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="D24" s="15" t="s">
         <v>6</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="H24" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="J24" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K24" s="11" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
     </row>
     <row r="25" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="D25" s="15" t="s">
         <v>6</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="J25" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K25" s="11" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="D26" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="H26" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="J26" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K26" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="D27" s="12" t="s">
         <v>5</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="H27" s="11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="J27" s="13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="K27" s="11" t="s">
-        <v>381</v>
+        <v>384</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:K4"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="44" customWidth="1"/>
+    <col min="2" max="2" width="70" customWidth="1"/>
+    <col min="3" max="3" width="50" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="16" t="s">
+        <v>566</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>567</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
+        <v>569</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>570</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="11" t="s">
+        <v>572</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>573</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>575</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
+        <v>577</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>578</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>580</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>581</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
+        <v>583</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>584</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="11" t="s">
+        <v>586</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>587</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>588</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K35"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="6" max="6" width="26" customWidth="1"/>
+    <col min="7" max="7" width="46" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
+    <col min="9" max="9" width="46" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+    </row>
+    <row r="2" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
+        <v>386</v>
+      </c>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
+        <v>387</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="K4" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
+        <v>388</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>389</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>390</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>391</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>392</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>395</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>396</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>397</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>400</v>
+      </c>
+      <c r="J6" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
+        <v>402</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>403</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>404</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>391</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>405</v>
+      </c>
+      <c r="J7" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="11" t="s">
+        <v>407</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>408</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>397</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>409</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>410</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>411</v>
+      </c>
+      <c r="J8" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="11" t="s">
+        <v>412</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>413</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>414</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>415</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>416</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>417</v>
+      </c>
+      <c r="J9" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
+        <v>419</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>420</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>421</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>422</v>
+      </c>
+      <c r="H10" s="11" t="s">
+        <v>423</v>
+      </c>
+      <c r="I10" s="11" t="s">
+        <v>424</v>
+      </c>
+      <c r="J10" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K10" s="11" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="H11" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I11" s="11" t="s">
+        <v>428</v>
+      </c>
+      <c r="J11" s="13" t="s">
+        <v>429</v>
+      </c>
+      <c r="K11" s="11" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
+        <v>431</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>433</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>434</v>
+      </c>
+      <c r="J12" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K12" s="11" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="11" t="s">
+        <v>436</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>437</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>438</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>439</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>440</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I13" s="11" t="s">
+        <v>441</v>
+      </c>
+      <c r="J13" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
+        <v>443</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>437</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>444</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>445</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>446</v>
+      </c>
+      <c r="H14" s="11" t="s">
+        <v>447</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>448</v>
+      </c>
+      <c r="J14" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K14" s="11" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
+        <v>449</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>437</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>450</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>451</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>446</v>
+      </c>
+      <c r="H15" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>452</v>
+      </c>
+      <c r="J15" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K15" s="11" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
+        <v>454</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>455</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>456</v>
+      </c>
+      <c r="G16" s="11" t="s">
+        <v>457</v>
+      </c>
+      <c r="H16" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I16" s="11" t="s">
+        <v>458</v>
+      </c>
+      <c r="J16" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K16" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
+        <v>459</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>460</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>461</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>462</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>463</v>
+      </c>
+      <c r="H17" s="11" t="s">
+        <v>464</v>
+      </c>
+      <c r="I17" s="11" t="s">
+        <v>465</v>
+      </c>
+      <c r="J17" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K17" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
+        <v>466</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>460</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>467</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>468</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I18" s="11" t="s">
+        <v>469</v>
+      </c>
+      <c r="J18" s="13" t="s">
+        <v>429</v>
+      </c>
+      <c r="K18" s="11" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="19" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
+        <v>471</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>472</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>473</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>474</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>475</v>
+      </c>
+      <c r="H19" s="11" t="s">
+        <v>476</v>
+      </c>
+      <c r="I19" s="11" t="s">
+        <v>477</v>
+      </c>
+      <c r="J19" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K19" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="11" t="s">
+        <v>478</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>472</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>479</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>480</v>
+      </c>
+      <c r="H20" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I20" s="11" t="s">
+        <v>481</v>
+      </c>
+      <c r="J20" s="13" t="s">
+        <v>429</v>
+      </c>
+      <c r="K20" s="11" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="11" t="s">
+        <v>483</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>484</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>485</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E21" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>486</v>
+      </c>
+      <c r="G21" s="11" t="s">
+        <v>487</v>
+      </c>
+      <c r="H21" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I21" s="11" t="s">
+        <v>488</v>
+      </c>
+      <c r="J21" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K21" s="11" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="11" t="s">
+        <v>490</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>484</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>491</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="G22" s="11" t="s">
+        <v>492</v>
+      </c>
+      <c r="H22" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I22" s="11" t="s">
+        <v>493</v>
+      </c>
+      <c r="J22" s="13" t="s">
+        <v>429</v>
+      </c>
+      <c r="K22" s="11" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="23" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="11" t="s">
+        <v>495</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>366</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>496</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E23" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F23" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="G23" s="11" t="s">
+        <v>497</v>
+      </c>
+      <c r="H23" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I23" s="11" t="s">
+        <v>498</v>
+      </c>
+      <c r="J23" s="13" t="s">
+        <v>429</v>
+      </c>
+      <c r="K23" s="11" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="24" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" s="11" t="s">
+        <v>500</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>366</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>501</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="G24" s="11" t="s">
+        <v>502</v>
+      </c>
+      <c r="H24" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I24" s="11" t="s">
+        <v>503</v>
+      </c>
+      <c r="J24" s="13" t="s">
+        <v>429</v>
+      </c>
+      <c r="K24" s="11" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="11" t="s">
+        <v>505</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>506</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>507</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E25" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F25" s="11" t="s">
+        <v>508</v>
+      </c>
+      <c r="G25" s="11" t="s">
+        <v>509</v>
+      </c>
+      <c r="H25" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I25" s="11" t="s">
+        <v>510</v>
+      </c>
+      <c r="J25" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K25" s="11" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="11" t="s">
+        <v>512</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>513</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E26" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F26" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="G26" s="11" t="s">
+        <v>514</v>
+      </c>
+      <c r="H26" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I26" s="11" t="s">
+        <v>515</v>
+      </c>
+      <c r="J26" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K26" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" s="11" t="s">
+        <v>516</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>517</v>
+      </c>
+      <c r="D27" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E27" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F27" s="11" t="s">
+        <v>518</v>
+      </c>
+      <c r="G27" s="11" t="s">
+        <v>519</v>
+      </c>
+      <c r="H27" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I27" s="11" t="s">
+        <v>520</v>
+      </c>
+      <c r="J27" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K27" s="11" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="11" t="s">
+        <v>522</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>523</v>
+      </c>
+      <c r="D28" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E28" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F28" s="11" t="s">
+        <v>357</v>
+      </c>
+      <c r="G28" s="11" t="s">
+        <v>524</v>
+      </c>
+      <c r="H28" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I28" s="11" t="s">
+        <v>525</v>
+      </c>
+      <c r="J28" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K28" s="11" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
+        <v>527</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>528</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E29" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F29" s="11" t="s">
+        <v>529</v>
+      </c>
+      <c r="G29" s="11" t="s">
+        <v>530</v>
+      </c>
+      <c r="H29" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I29" s="11" t="s">
+        <v>531</v>
+      </c>
+      <c r="J29" s="13" t="s">
+        <v>429</v>
+      </c>
+      <c r="K29" s="11" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="30" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="11" t="s">
+        <v>533</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>534</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E30" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F30" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>535</v>
+      </c>
+      <c r="H30" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I30" s="11" t="s">
+        <v>536</v>
+      </c>
+      <c r="J30" s="13" t="s">
+        <v>429</v>
+      </c>
+      <c r="K30" s="11" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="11" t="s">
+        <v>538</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>539</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E31" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="F31" s="11" t="s">
+        <v>508</v>
+      </c>
+      <c r="G31" s="11" t="s">
+        <v>540</v>
+      </c>
+      <c r="H31" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I31" s="11" t="s">
+        <v>541</v>
+      </c>
+      <c r="J31" s="13" t="s">
+        <v>429</v>
+      </c>
+      <c r="K31" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="32" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="11" t="s">
+        <v>542</v>
+      </c>
+      <c r="B32" s="11" t="s">
+        <v>543</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>544</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E32" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F32" s="11" t="s">
+        <v>545</v>
+      </c>
+      <c r="G32" s="11" t="s">
+        <v>546</v>
+      </c>
+      <c r="H32" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I32" s="11" t="s">
+        <v>547</v>
+      </c>
+      <c r="J32" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K32" s="11" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="33" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="11" t="s">
+        <v>549</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>550</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>551</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E33" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F33" s="11" t="s">
+        <v>552</v>
+      </c>
+      <c r="G33" s="11" t="s">
+        <v>553</v>
+      </c>
+      <c r="H33" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I33" s="11" t="s">
+        <v>554</v>
+      </c>
+      <c r="J33" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K33" s="11" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="11" t="s">
+        <v>556</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>550</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>557</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E34" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="G34" s="11" t="s">
+        <v>558</v>
+      </c>
+      <c r="H34" s="11" t="s">
+        <v>559</v>
+      </c>
+      <c r="I34" s="11" t="s">
+        <v>560</v>
+      </c>
+      <c r="J34" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K34" s="11" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="11" t="s">
+        <v>562</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>376</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>563</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E35" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="F35" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="G35" s="11" t="s">
+        <v>564</v>
+      </c>
+      <c r="H35" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I35" s="11" t="s">
+        <v>565</v>
+      </c>
+      <c r="J35" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="K35" s="11" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -4199,75 +6104,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="44" customWidth="1"/>
-    <col min="2" max="2" width="70" customWidth="1"/>
-    <col min="3" max="3" width="50" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
-        <v>382</v>
-      </c>
-      <c r="B1" s="16" t="s">
-        <v>383</v>
-      </c>
-      <c r="C1" s="16" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
-        <v>385</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>386</v>
-      </c>
-      <c r="C2" s="11" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
-        <v>388</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>389</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>391</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
-        <v>393</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>394</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>395</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix coverage gaps: PDI lists all vehicles, Enquiry dates, config cleanup
- PDI: raise the page's "Top" box (25 by default) to PDI_TOP (500) and
  click Show before reading the grid; warn if the list is full. D71001
  went from 25 to 28 vehicles and 10 to 11 blank chassis.
- Enquiry List: report dates from ENQ_FROM / ENQ_TO (dd-mm-yyyy); the
  default is unchanged (07-09-2026 to today).
- playwright.config.ts: drop the setup and enroll-passkey projects and
  the saved-login file; no such files exist and every spec logs in.
- PDI dry-run result lines count filled chassis instead of "0 updated".
- Test cases: email cases removed from the PDI sheet; wrong login, not
  in VIN sheet, Top N and PDI_TOP cases run and passed; ENQ-16/17 added;
  Summary recounted from the sheets; fixed coverage gaps marked.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Test Cases/DMS_Automation_Test_Cases.xlsx
+++ b/Test Cases/DMS_Automation_Test_Cases.xlsx
@@ -16,12 +16,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1073" uniqueCount="589">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="591">
   <si>
     <t>River DMS - E2E Automation Test Cases</t>
   </si>
   <si>
-    <t>Enquiry List, GSTR and MIS test cases executed on 25-Sep-2026; PDI Vehicle Details on 28-Sep-2026 — all against the live DMS (Microsoft Edge and Google Chrome). "Not run yet" = handled in code, not yet seen in a live run.</t>
+    <t>Enquiry List, GSTR and MIS test cases executed on 25-Sep-2026; PDI Vehicle Details and ENQ-16/17 on 28-Sep-2026 — all against the live DMS (Microsoft Edge and Google Chrome). "Not run yet" = handled in code, not yet seen in a live run.</t>
   </si>
   <si>
     <t>Sheet</t>
@@ -440,6 +440,48 @@
     <t>CREDENTIALS_FILE pointed to a copy of credentials.json; logged in and passed in 55s</t>
   </si>
   <si>
+    <t>ENQ-16</t>
+  </si>
+  <si>
+    <t>Report dates from settings</t>
+  </si>
+  <si>
+    <t>ENQ_FROM / ENQ_TO set</t>
+  </si>
+  <si>
+    <t>ENQ_FROM=20-09-2026 ENQ_TO=27-09-2026 npx playwright test tests/enquiryListReport.spec.ts</t>
+  </si>
+  <si>
+    <t>ENQ_FROM=20-09-2026, ENQ_TO=27-09-2026</t>
+  </si>
+  <si>
+    <t>All three reports use that range</t>
+  </si>
+  <si>
+    <t>Pass (28-Sep-2026)</t>
+  </si>
+  <si>
+    <t>Passed in 46 s: 10,596 enquiries / 1,361 invoices / 1,815 bookings</t>
+  </si>
+  <si>
+    <t>ENQ-17</t>
+  </si>
+  <si>
+    <t>Date setting in the wrong format</t>
+  </si>
+  <si>
+    <t>ENQ_FROM=2026/09/01</t>
+  </si>
+  <si>
+    <t>Run the test</t>
+  </si>
+  <si>
+    <t>Stops at once: "ENQ_FROM must be dd-mm-yyyy"</t>
+  </si>
+  <si>
+    <t>Exact message seen</t>
+  </si>
+  <si>
     <t>GSTR Report - tests/GSTR Report.spec.ts</t>
   </si>
   <si>
@@ -495,9 +537,6 @@
   </si>
   <si>
     <t>One dealer with a bad password</t>
-  </si>
-  <si>
-    <t>Run the test</t>
   </si>
   <si>
     <t>"Login failed: still on the login page" logged; screenshot attached; dealer retried once at the end; other dealers complete; MasterData saved; test marked failed listing that dealer</t>
@@ -821,9 +860,6 @@
     <t>GSTR-23</t>
   </si>
   <si>
-    <t>Date setting in the wrong format</t>
-  </si>
-  <si>
     <t>GSTR_FROM=2026/09/01</t>
   </si>
   <si>
@@ -1196,7 +1232,7 @@
     <t>PDI Vehicle Details - tests/PDI.spec.ts</t>
   </si>
   <si>
-    <t>For every dealer in PIDUsers: find WORKSHOP &gt; PDI rows with a blank field, fill Engine / Battery / Charger from the VIN Details sheet in SETTINGS &gt; Admin &gt; Modify vehicle details, Save and confirm; per-dealer report emailed (CC) only when the run fully passes, plus a daily combined report.</t>
+    <t>For every dealer in PIDUsers: find WORKSHOP &gt; PDI rows with a blank field (all vehicles, not just the top 25), fill Engine / Battery / Charger from the VIN Details sheet in SETTINGS &gt; Admin &gt; Modify vehicle details, Save and confirm; per-dealer results in Output, plus a daily combined report.</t>
   </si>
   <si>
     <t>Run: npm run test:pdi   (dry run: npm run test:pdi:dry, daily report: npm run report:pdi-daily)</t>
@@ -1217,9 +1253,6 @@
     <t>Stops before any login, naming the dealer(s); nothing is changed</t>
   </si>
   <si>
-    <t>Pass (28-Sep-2026)</t>
-  </si>
-  <si>
     <t>292006 with &lt;user&gt;/&lt;password&gt;: stopped at once (message wording from an earlier build)</t>
   </si>
   <si>
@@ -1277,6 +1310,21 @@
     <t>PDI-05</t>
   </si>
   <si>
+    <t>PDI_TOP is not a number</t>
+  </si>
+  <si>
+    <t>PDI_TOP=abc npx playwright test tests/PDI.spec.ts</t>
+  </si>
+  <si>
+    <t>PDI_TOP=abc</t>
+  </si>
+  <si>
+    <t>Stops at once: "PDI_TOP must be a whole number above 0"</t>
+  </si>
+  <si>
+    <t>PDI-06</t>
+  </si>
+  <si>
     <t>Safety</t>
   </si>
   <si>
@@ -1289,13 +1337,13 @@
     <t>npx playwright test tests/PDI.spec.ts tests/PDIDailyReport.spec.ts</t>
   </si>
   <si>
-    <t>Both specs skipped — no DMS changes, no email</t>
+    <t>Both specs skipped — no DMS changes</t>
   </si>
   <si>
     <t>"2 skipped"</t>
   </si>
   <si>
-    <t>PDI-06</t>
+    <t>PDI-07</t>
   </si>
   <si>
     <t>Each PIDUsers dealer logs in</t>
@@ -1316,142 +1364,172 @@
     <t>15/15 dealers across the 28-Sep runs</t>
   </si>
   <si>
-    <t>PDI-07</t>
-  </si>
-  <si>
-    <t>Run with several dealers</t>
-  </si>
-  <si>
-    <t>That dealer marked failed (screenshot attached); other dealers still run; test red; no report email</t>
+    <t>PDI-08</t>
+  </si>
+  <si>
+    <t>Wrong login for one dealer</t>
+  </si>
+  <si>
+    <t>One dealer with a bad login</t>
+  </si>
+  <si>
+    <t>Run with several dealers (dry run)</t>
+  </si>
+  <si>
+    <t>Scratch credentials: D71001 + fake dealer 999998</t>
+  </si>
+  <si>
+    <t>That dealer marked failed (screenshot attached); other dealers still run; test red</t>
+  </si>
+  <si>
+    <t>999998: "Login failed: still on the login page"; D71001 still processed; run red with both problems listed</t>
+  </si>
+  <si>
+    <t>PDI-09</t>
+  </si>
+  <si>
+    <t>Open WORKSHOP &gt; PDI</t>
+  </si>
+  <si>
+    <t>Click WORKSHOP, then PDI (matched by link, as menu names carry an icon)</t>
+  </si>
+  <si>
+    <t>PDI grid (PDIStockCheckingMain.aspx) is shown</t>
+  </si>
+  <si>
+    <t>Worked for all dealers</t>
+  </si>
+  <si>
+    <t>PDI-10</t>
+  </si>
+  <si>
+    <t>PDI grid</t>
+  </si>
+  <si>
+    <t>List every vehicle, not just the top 25</t>
+  </si>
+  <si>
+    <t>PDI page open</t>
+  </si>
+  <si>
+    <t>Set "Top" to PDI_TOP (500) and click Show before reading the grid</t>
+  </si>
+  <si>
+    <t>PDI_TOP=500 (default)</t>
+  </si>
+  <si>
+    <t>All vehicles listed; WARN if the list is full</t>
+  </si>
+  <si>
+    <t>D71001: 25 -&gt; 28 vehicles, 10 -&gt; 11 blank (one blank chassis had been hidden)</t>
+  </si>
+  <si>
+    <t>PDI-11</t>
+  </si>
+  <si>
+    <t>Rows with a blank field are found</t>
+  </si>
+  <si>
+    <t>PDI grid loaded</t>
+  </si>
+  <si>
+    <t>Read inputs //input[starts-with(@id,"ctl00_cpMain_grdMain_")], group by row, keep rows with any empty field and save their ChassisNo</t>
+  </si>
+  <si>
+    <t>Chassis numbers listed with the blank field names</t>
+  </si>
+  <si>
+    <t>EngineNo was the blank field on every dealer</t>
+  </si>
+  <si>
+    <t>PDI-12</t>
+  </si>
+  <si>
+    <t>PDI grid is empty</t>
+  </si>
+  <si>
+    <t>Dealer with no vehicles waiting for PDI</t>
+  </si>
+  <si>
+    <t>Open PDI</t>
+  </si>
+  <si>
+    <t>271001</t>
+  </si>
+  <si>
+    <t>"PDI grid is empty", "Nothing to update"; Modify page not opened</t>
+  </si>
+  <si>
+    <t>PDI-13</t>
+  </si>
+  <si>
+    <t>No blank rows</t>
+  </si>
+  <si>
+    <t>Every PDI row filled</t>
+  </si>
+  <si>
+    <t>"0 PDI row(s) with blank fields", "Nothing to update"</t>
+  </si>
+  <si>
+    <t>e.g. 292005, 292010, and dealers re-checked after being updated</t>
+  </si>
+  <si>
+    <t>PDI-14</t>
+  </si>
+  <si>
+    <t>Open SETTINGS &gt; Admin &gt; Modify vehicle details</t>
+  </si>
+  <si>
+    <t>Blank rows found</t>
+  </si>
+  <si>
+    <t>SETTINGS &gt; Admin &gt; Modify vehicle details</t>
+  </si>
+  <si>
+    <t>ChangeChassisNo.aspx is shown</t>
+  </si>
+  <si>
+    <t>PDI-15</t>
+  </si>
+  <si>
+    <t>Modify vehicle</t>
+  </si>
+  <si>
+    <t>Show loads the chassis</t>
+  </si>
+  <si>
+    <t>Modify page open</t>
+  </si>
+  <si>
+    <t>Enter chassis in ctl00$cpMain$IdentifierValue, click Show, wait 10 s</t>
+  </si>
+  <si>
+    <t>Chassis from the PDI grid</t>
+  </si>
+  <si>
+    <t>Form shows the same ChassisNo</t>
+  </si>
+  <si>
+    <t>PDI-16</t>
+  </si>
+  <si>
+    <t>Show loads a different vehicle / nothing</t>
+  </si>
+  <si>
+    <t>Show a chassis the DMS can't find</t>
+  </si>
+  <si>
+    <t>Skipped: "Show did not load this vehicle"; nothing saved; test red</t>
   </si>
   <si>
     <t>Not run yet</t>
   </si>
   <si>
-    <t>Handled by the per-dealer try/catch; not yet run against the DMS</t>
-  </si>
-  <si>
-    <t>PDI-08</t>
-  </si>
-  <si>
-    <t>Open WORKSHOP &gt; PDI</t>
-  </si>
-  <si>
-    <t>Click WORKSHOP, then PDI (matched by link, as menu names carry an icon)</t>
-  </si>
-  <si>
-    <t>PDI grid (PDIStockCheckingMain.aspx) is shown</t>
-  </si>
-  <si>
-    <t>Worked for all 15 dealers</t>
-  </si>
-  <si>
-    <t>PDI-09</t>
-  </si>
-  <si>
-    <t>PDI grid</t>
-  </si>
-  <si>
-    <t>Rows with a blank field are found</t>
-  </si>
-  <si>
-    <t>PDI grid loaded</t>
-  </si>
-  <si>
-    <t>Read inputs //input[starts-with(@id,"ctl00_cpMain_grdMain_")], group by row, keep rows with any empty field and save their ChassisNo</t>
-  </si>
-  <si>
-    <t>Chassis numbers listed with the blank field names</t>
-  </si>
-  <si>
-    <t>EngineNo was the blank field on every dealer</t>
-  </si>
-  <si>
-    <t>PDI-10</t>
-  </si>
-  <si>
-    <t>PDI grid is empty</t>
-  </si>
-  <si>
-    <t>Dealer with no vehicles waiting for PDI</t>
-  </si>
-  <si>
-    <t>Open PDI</t>
-  </si>
-  <si>
-    <t>271001</t>
-  </si>
-  <si>
-    <t>"PDI grid is empty", "Nothing to update"; Modify page not opened</t>
-  </si>
-  <si>
-    <t>PDI-11</t>
-  </si>
-  <si>
-    <t>No blank rows</t>
-  </si>
-  <si>
-    <t>Every PDI row filled</t>
-  </si>
-  <si>
-    <t>"0 PDI row(s) with blank fields", "Nothing to update"</t>
-  </si>
-  <si>
-    <t>e.g. 292005, 292010, and dealers re-checked after being updated</t>
-  </si>
-  <si>
-    <t>PDI-12</t>
-  </si>
-  <si>
-    <t>Open SETTINGS &gt; Admin &gt; Modify vehicle details</t>
-  </si>
-  <si>
-    <t>Blank rows found</t>
-  </si>
-  <si>
-    <t>SETTINGS &gt; Admin &gt; Modify vehicle details</t>
-  </si>
-  <si>
-    <t>ChangeChassisNo.aspx is shown</t>
-  </si>
-  <si>
-    <t>PDI-13</t>
-  </si>
-  <si>
-    <t>Modify vehicle</t>
-  </si>
-  <si>
-    <t>Show loads the chassis</t>
-  </si>
-  <si>
-    <t>Modify page open</t>
-  </si>
-  <si>
-    <t>Enter chassis in ctl00$cpMain$IdentifierValue, click Show, wait 10 s</t>
-  </si>
-  <si>
-    <t>Chassis from PDI-09</t>
-  </si>
-  <si>
-    <t>Form shows the same ChassisNo</t>
-  </si>
-  <si>
-    <t>PDI-14</t>
-  </si>
-  <si>
-    <t>Show loads a different vehicle / nothing</t>
-  </si>
-  <si>
-    <t>Show a chassis the DMS can't find</t>
-  </si>
-  <si>
-    <t>Skipped: "Show did not load this vehicle"; nothing saved; test red</t>
-  </si>
-  <si>
     <t>Handled in code; no such chassis met yet</t>
   </si>
   <si>
-    <t>PDI-15</t>
+    <t>PDI-17</t>
   </si>
   <si>
     <t>VIN lookup</t>
@@ -1472,22 +1550,25 @@
     <t>All four fields filled with the sheet's values</t>
   </si>
   <si>
-    <t>PDI-16</t>
+    <t>PDI-18</t>
   </si>
   <si>
     <t>Chassis not in the VIN Details sheet</t>
   </si>
   <si>
-    <t>Run with a chassis missing from the sheet</t>
-  </si>
-  <si>
-    <t>Skipped and listed as "Not in VIN Details sheet"; test red; no report email</t>
-  </si>
-  <si>
-    <t>Every chassis on 28-Sep was in the sheet; shown correctly in the dashboard preview with sample data</t>
-  </si>
-  <si>
-    <t>PDI-17</t>
+    <t>Run with a chassis missing from the sheet (dry run)</t>
+  </si>
+  <si>
+    <t>Copy of the VIN sheet without P7BAABXX1JT059691</t>
+  </si>
+  <si>
+    <t>Skipped and listed as "Not in VIN Details sheet"; other chassis continue; test red</t>
+  </si>
+  <si>
+    <t>D71001: P7BAABXX1JT059691 skipped and listed; run red</t>
+  </si>
+  <si>
+    <t>PDI-19</t>
   </si>
   <si>
     <t>Save</t>
@@ -1508,7 +1589,7 @@
     <t>160 chassis updated across 12 dealers on 28-Sep</t>
   </si>
   <si>
-    <t>PDI-18</t>
+    <t>PDI-20</t>
   </si>
   <si>
     <t>Save clicked but the values were not kept</t>
@@ -1517,13 +1598,13 @@
     <t>DMS rejects or ignores the change</t>
   </si>
   <si>
-    <t>"Save clicked but values not kept"; test red; no report email</t>
+    <t>"Save clicked but values not kept"; test red</t>
   </si>
   <si>
     <t>Handled in code; not seen yet</t>
   </si>
   <si>
-    <t>PDI-19</t>
+    <t>PDI-21</t>
   </si>
   <si>
     <t>Page times out mid-dealer: recover and retry</t>
@@ -1538,7 +1619,7 @@
     <t>Added after 4 timeouts on 372002 (13:38 run). Those 4 were checked in the DMS afterwards: values match the VIN sheet</t>
   </si>
   <si>
-    <t>PDI-20</t>
+    <t>PDI-22</t>
   </si>
   <si>
     <t>Page cannot be recovered</t>
@@ -1553,7 +1634,7 @@
     <t>Handled in code</t>
   </si>
   <si>
-    <t>PDI-21</t>
+    <t>PDI-23</t>
   </si>
   <si>
     <t>Dry run</t>
@@ -1568,13 +1649,13 @@
     <t>npm run test:pdi:dry</t>
   </si>
   <si>
-    <t>Form filled for every blank chassis, Save never clicked; report marked DRY RUN</t>
-  </si>
-  <si>
-    <t>D71001: 10 chassis filled, nothing saved</t>
-  </si>
-  <si>
-    <t>PDI-22</t>
+    <t>Form filled for every blank chassis, Save never clicked</t>
+  </si>
+  <si>
+    <t>D71001: 10 filled (morning run); 10 of 11 filled + 1 not in VIN sheet (negative test); nothing saved</t>
+  </si>
+  <si>
+    <t>PDI-24</t>
   </si>
   <si>
     <t>Results Excel with a Dealers sheet</t>
@@ -1586,7 +1667,7 @@
     <t>Output/PDI_BlankChassis_&lt;time&gt;.xlsx: one row per chassis + every dealer checked</t>
   </si>
   <si>
-    <t>PDI-23</t>
+    <t>PDI-25</t>
   </si>
   <si>
     <t>Results Excel is open in Excel (locked)</t>
@@ -1601,114 +1682,54 @@
     <t>Saved beside it as &lt;name&gt;_&lt;timestamp&gt;.xlsx; run continues</t>
   </si>
   <si>
-    <t>Locked PDI_Daily_2026-09-28.xlsx: EBUSY -&gt; saved as _1790610722383.xlsx, report still built</t>
-  </si>
-  <si>
-    <t>PDI-24</t>
-  </si>
-  <si>
-    <t>Report email with dashboard and Excel</t>
-  </si>
-  <si>
-    <t>Passing run ends</t>
-  </si>
-  <si>
-    <t>HTML summary per dealer in the body; PDI_Dashboard.html and the Excel attached</t>
-  </si>
-  <si>
-    <t>Emailed on 28-Sep (before the CC list was added)</t>
-  </si>
-  <si>
-    <t>PDI-25</t>
-  </si>
-  <si>
-    <t>CC list on a passing run</t>
-  </si>
-  <si>
-    <t>PDI_CC in .env</t>
-  </si>
-  <si>
-    <t>Passing real (not dry) run ends</t>
-  </si>
-  <si>
-    <t>Email goes to GMAIL_TO with the PDI_CC people on CC</t>
-  </si>
-  <si>
-    <t>Rule checked with data; the first CC email will be the next passing run</t>
+    <t>Locked PDI_Daily_2026-09-28.xlsx: EBUSY -&gt; saved as _1790610722383.xlsx, run passed</t>
   </si>
   <si>
     <t>PDI-26</t>
   </si>
   <si>
-    <t>Failed run sends no report</t>
-  </si>
-  <si>
-    <t>Run with any timeout, missing VIN, values not kept, or failed dealer</t>
-  </si>
-  <si>
-    <t>No PDI report emailed to anyone; test red; dashboard and Excel still saved</t>
-  </si>
-  <si>
-    <t>Rule checked with sample data (1 timeout / failed login / not in VIN sheet -&gt; not sent); not yet seen in a live run</t>
+    <t>Dashboard</t>
+  </si>
+  <si>
+    <t>Interactive dashboard</t>
+  </si>
+  <si>
+    <t>PDI_Dashboard.html (saved in Output)</t>
+  </si>
+  <si>
+    <t>Open in a browser; click a dealer bar, outcome chips, search, sort columns, theme toggle, phone width</t>
+  </si>
+  <si>
+    <t>Table filters / sorts correctly; dark mode and phone layout work</t>
+  </si>
+  <si>
+    <t>Sample data: dealer + Error filter -&gt; "2 of 14"; no script errors; no sideways scroll at 390 px</t>
   </si>
   <si>
     <t>PDI-27</t>
   </si>
   <si>
-    <t>Dry-run report goes only to GMAIL_TO</t>
-  </si>
-  <si>
-    <t>Dry run ends</t>
-  </si>
-  <si>
-    <t>Email marked DRY RUN, no CC</t>
+    <t>Daily report</t>
+  </si>
+  <si>
+    <t>Combine the day's runs</t>
+  </si>
+  <si>
+    <t>Result files in Output</t>
+  </si>
+  <si>
+    <t>npm run report:pdi-daily</t>
+  </si>
+  <si>
+    <t>Latest result per chassis; dry runs left out; errors cleared by a later check shown as Updated</t>
+  </si>
+  <si>
+    <t>28-Sep: 5 runs -&gt; 160 chassis, 15 dealers; 372002's 4 timeouts shown as Updated</t>
   </si>
   <si>
     <t>PDI-28</t>
   </si>
   <si>
-    <t>Dashboard</t>
-  </si>
-  <si>
-    <t>Interactive dashboard</t>
-  </si>
-  <si>
-    <t>PDI_Dashboard.html</t>
-  </si>
-  <si>
-    <t>Open in a browser; click a dealer bar, outcome chips, search, sort columns, theme toggle, phone width</t>
-  </si>
-  <si>
-    <t>Table filters / sorts correctly; dark mode and phone layout work</t>
-  </si>
-  <si>
-    <t>Sample data: dealer + Error filter -&gt; "2 of 14"; no script errors; no sideways scroll at 390 px</t>
-  </si>
-  <si>
-    <t>PDI-29</t>
-  </si>
-  <si>
-    <t>Daily report</t>
-  </si>
-  <si>
-    <t>Combine the day's runs into one report</t>
-  </si>
-  <si>
-    <t>Result files in Output</t>
-  </si>
-  <si>
-    <t>npm run report:pdi-daily</t>
-  </si>
-  <si>
-    <t>Latest result per chassis; dry runs left out; errors cleared by a later check shown as Updated</t>
-  </si>
-  <si>
-    <t>28-Sep: 5 runs -&gt; 160 chassis, 15 dealers; 372002's 4 timeouts shown as Updated</t>
-  </si>
-  <si>
-    <t>PDI-30</t>
-  </si>
-  <si>
     <t>No runs on that day</t>
   </si>
   <si>
@@ -1721,21 +1742,6 @@
     <t>Stops: "No PDI result files from 2020-01-01"</t>
   </si>
   <si>
-    <t>Exact message seen</t>
-  </si>
-  <si>
-    <t>PDI-31</t>
-  </si>
-  <si>
-    <t>Build the report without emailing</t>
-  </si>
-  <si>
-    <t>PDI_SEND_EMAIL=0</t>
-  </si>
-  <si>
-    <t>"report email skipped"; dashboard and Excel still saved</t>
-  </si>
-  <si>
     <t>Item</t>
   </si>
   <si>
@@ -1760,13 +1766,13 @@
     <t>Matches *.setup.ts but no such file exists; "Google Chrome" project expects playwright/.auth/salesforce.json (both specs override it with an empty session)</t>
   </si>
   <si>
-    <t>Remove the setup dependency / storageState, or add a setup file</t>
+    <t>Fixed (28-Sep-2026): setup and enroll-passkey projects and the unused saved-login file removed from playwright.config.ts; Enquiry List passed with the new config</t>
   </si>
   <si>
     <t>From date hard-coded to 7 Sep 2026</t>
   </si>
   <si>
-    <t>Make the date configurable like GSTR_FROM / GSTR_TO</t>
+    <t>Fixed (28-Sep-2026): ENQ_FROM / ENQ_TO (dd-mm-yyyy), default unchanged (07-09-2026 to today) — see ENQ-16 / ENQ-17</t>
   </si>
   <si>
     <t>CI/CD (.github/workflows/playwright.yml)</t>
@@ -1775,7 +1781,7 @@
     <t>Not yet run on GitHub Actions; needs repository secrets CREDENTIALS_JSON, GMAIL_USER, GMAIL_APP_PASSWORD, GMAIL_TO</t>
   </si>
   <si>
-    <t>Add the secrets, then run the workflow manually once</t>
+    <t>Needs the repository owner: add the secrets under Settings &gt; Secrets and variables &gt; Actions, then run the workflow once (cannot be done from this PC — no GitHub CLI / secret values are private)</t>
   </si>
   <si>
     <t>tests/PDI.spec.ts — PDI grid size</t>
@@ -1784,13 +1790,13 @@
     <t>Only the rows the PDI page shows are checked (Top N = 25 by default); blank rows further down are missed</t>
   </si>
   <si>
-    <t>Set the Top N box higher before reading the grid if a dealer can have more than 25 vehicles waiting</t>
+    <t>Fixed (28-Sep-2026): the spec sets "Top" to PDI_TOP (500) and clicks Show; warns if the list is full — see the "top 25" PDI case</t>
   </si>
   <si>
     <t>tests/PDI.spec.ts — not yet run live</t>
   </si>
   <si>
-    <t>PDI-07, 14, 16, 18, 19, 20, 25, 26, 27 are handled in code but have not happened in a real run yet</t>
+    <t>PDI-16, PDI-20, PDI-21, PDI-22 are handled in code but have not happened in a real run yet</t>
   </si>
   <si>
     <t>Mark them Pass the first time each one is seen</t>
@@ -2348,19 +2354,19 @@
         <v>11</v>
       </c>
       <c r="C5" s="5">
+        <v>16</v>
+      </c>
+      <c r="D5" s="5">
         <v>14</v>
       </c>
-      <c r="D5" s="5">
-        <v>13</v>
-      </c>
       <c r="E5" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="5">
         <v>1</v>
       </c>
       <c r="G5" s="5">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>12</v>
@@ -2426,19 +2432,19 @@
         <v>20</v>
       </c>
       <c r="C8" s="5">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D8" s="5">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E8" s="5">
         <v>12</v>
       </c>
       <c r="F8" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G8" s="5">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>21</v>
@@ -2452,19 +2458,19 @@
         <v>22</v>
       </c>
       <c r="C9" s="6">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D9" s="6">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E9" s="6">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F9" s="6">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G9" s="6">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>22</v>
@@ -2488,7 +2494,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -3071,6 +3077,76 @@
       </c>
       <c r="K18" s="11" t="s">
         <v>135</v>
+      </c>
+    </row>
+    <row r="19" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="H19" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="I19" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="J19" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="K19" s="11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="H20" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I20" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="J20" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="K20" s="11" t="s">
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -3104,7 +3180,7 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>136</v>
+        <v>150</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -3119,7 +3195,7 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -3134,7 +3210,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -3184,13 +3260,13 @@
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>130</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>6</v>
@@ -3199,33 +3275,33 @@
         <v>40</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>143</v>
+        <v>157</v>
       </c>
       <c r="J5" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K5" s="11" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>38</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>5</v>
@@ -3234,33 +3310,33 @@
         <v>40</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>147</v>
+        <v>161</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>148</v>
+        <v>162</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
       <c r="J6" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="B7" s="11" t="s">
         <v>38</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>153</v>
+        <v>167</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>6</v>
@@ -3269,33 +3345,33 @@
         <v>40</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="H7" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="J7" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K7" s="11" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>48</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>5</v>
@@ -3307,13 +3383,13 @@
         <v>50</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="H8" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="J8" s="13" t="s">
         <v>45</v>
@@ -3324,13 +3400,13 @@
     </row>
     <row r="9" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>54</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="D9" s="12" t="s">
         <v>5</v>
@@ -3339,16 +3415,16 @@
         <v>40</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="J9" s="13" t="s">
         <v>45</v>
@@ -3359,13 +3435,13 @@
     </row>
     <row r="10" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>54</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>7</v>
@@ -3374,33 +3450,33 @@
         <v>83</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="H10" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="J10" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K10" s="11" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="D11" s="12" t="s">
         <v>5</v>
@@ -3409,16 +3485,16 @@
         <v>40</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="J11" s="13" t="s">
         <v>45</v>
@@ -3429,13 +3505,13 @@
     </row>
     <row r="12" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="D12" s="14" t="s">
         <v>7</v>
@@ -3444,33 +3520,33 @@
         <v>40</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="J12" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K12" s="11" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>188</v>
       </c>
-      <c r="B13" s="11" t="s">
-        <v>175</v>
-      </c>
       <c r="C13" s="11" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="D13" s="14" t="s">
         <v>7</v>
@@ -3479,33 +3555,33 @@
         <v>83</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="H13" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="J13" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K13" s="11" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>5</v>
@@ -3514,33 +3590,33 @@
         <v>40</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="J14" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="D15" s="14" t="s">
         <v>7</v>
@@ -3549,33 +3625,33 @@
         <v>83</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="J15" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="D16" s="12" t="s">
         <v>5</v>
@@ -3584,33 +3660,33 @@
         <v>40</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>213</v>
+        <v>226</v>
       </c>
       <c r="H16" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
       <c r="J16" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K16" s="11" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="D17" s="12" t="s">
         <v>5</v>
@@ -3619,33 +3695,33 @@
         <v>40</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>219</v>
+        <v>232</v>
       </c>
       <c r="H17" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="J17" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K17" s="11" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
     </row>
     <row r="18" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="D18" s="14" t="s">
         <v>7</v>
@@ -3654,33 +3730,33 @@
         <v>40</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="H18" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="J18" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K18" s="11" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>6</v>
@@ -3689,33 +3765,33 @@
         <v>83</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="H19" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
       <c r="J19" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K19" s="11" t="s">
-        <v>233</v>
+        <v>246</v>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>235</v>
+        <v>248</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>236</v>
+        <v>249</v>
       </c>
       <c r="D20" s="12" t="s">
         <v>5</v>
@@ -3724,16 +3800,16 @@
         <v>83</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>237</v>
+        <v>250</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="H20" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
       <c r="J20" s="13" t="s">
         <v>45</v>
@@ -3744,13 +3820,13 @@
     </row>
     <row r="21" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>241</v>
+        <v>254</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>6</v>
@@ -3759,33 +3835,33 @@
         <v>40</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>243</v>
+        <v>256</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="H21" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>244</v>
+        <v>257</v>
       </c>
       <c r="J21" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K21" s="11" t="s">
-        <v>245</v>
+        <v>258</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>247</v>
+        <v>260</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="D22" s="12" t="s">
         <v>5</v>
@@ -3794,33 +3870,33 @@
         <v>40</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>249</v>
+        <v>262</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>250</v>
+        <v>263</v>
       </c>
       <c r="H22" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>251</v>
+        <v>264</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K22" s="11" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>253</v>
+        <v>266</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>130</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>254</v>
+        <v>267</v>
       </c>
       <c r="D23" s="12" t="s">
         <v>5</v>
@@ -3829,33 +3905,33 @@
         <v>83</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>257</v>
+        <v>270</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>258</v>
+        <v>271</v>
       </c>
       <c r="J23" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K23" s="11" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>260</v>
+        <v>273</v>
       </c>
       <c r="B24" s="11" t="s">
         <v>130</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>261</v>
+        <v>145</v>
       </c>
       <c r="D24" s="15" t="s">
         <v>6</v>
@@ -3864,22 +3940,22 @@
         <v>104</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>262</v>
+        <v>274</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="H24" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="J24" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K24" s="11" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
     </row>
   </sheetData>
@@ -3913,7 +3989,7 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -3928,7 +4004,7 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -3943,7 +4019,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>267</v>
+        <v>279</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -3993,13 +4069,13 @@
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>38</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>5</v>
@@ -4008,16 +4084,16 @@
         <v>40</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>270</v>
+        <v>282</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="J5" s="13" t="s">
         <v>45</v>
@@ -4028,13 +4104,13 @@
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>38</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>6</v>
@@ -4043,33 +4119,33 @@
         <v>40</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>275</v>
+        <v>287</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>276</v>
+        <v>288</v>
       </c>
       <c r="H6" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
       <c r="J6" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>278</v>
+        <v>290</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>279</v>
+        <v>291</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>280</v>
+        <v>292</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>281</v>
+        <v>293</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>5</v>
@@ -4081,30 +4157,30 @@
         <v>50</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>282</v>
+        <v>294</v>
       </c>
       <c r="H7" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="J7" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K7" s="11" t="s">
-        <v>284</v>
+        <v>296</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>285</v>
+        <v>297</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>54</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>5</v>
@@ -4116,30 +4192,30 @@
         <v>22</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>287</v>
+        <v>299</v>
       </c>
       <c r="H8" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="J8" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>289</v>
+        <v>301</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>291</v>
+        <v>303</v>
       </c>
       <c r="D9" s="12" t="s">
         <v>5</v>
@@ -4151,13 +4227,13 @@
         <v>22</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>292</v>
+        <v>304</v>
       </c>
       <c r="H9" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>293</v>
+        <v>305</v>
       </c>
       <c r="J9" s="13" t="s">
         <v>45</v>
@@ -4168,13 +4244,13 @@
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>295</v>
+        <v>307</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>7</v>
@@ -4186,30 +4262,30 @@
         <v>22</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>292</v>
+        <v>304</v>
       </c>
       <c r="H10" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="J10" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K10" s="11" t="s">
-        <v>297</v>
+        <v>309</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>298</v>
+        <v>310</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>299</v>
+        <v>311</v>
       </c>
       <c r="D11" s="15" t="s">
         <v>6</v>
@@ -4221,30 +4297,30 @@
         <v>22</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>292</v>
+        <v>304</v>
       </c>
       <c r="H11" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="J11" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K11" s="11" t="s">
-        <v>301</v>
+        <v>313</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
+        <v>314</v>
+      </c>
+      <c r="B12" s="11" t="s">
         <v>302</v>
       </c>
-      <c r="B12" s="11" t="s">
-        <v>290</v>
-      </c>
       <c r="C12" s="11" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="D12" s="15" t="s">
         <v>6</v>
@@ -4253,33 +4329,33 @@
         <v>40</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>305</v>
+        <v>317</v>
       </c>
       <c r="H12" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>306</v>
+        <v>318</v>
       </c>
       <c r="J12" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K12" s="11" t="s">
-        <v>307</v>
+        <v>319</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>308</v>
+        <v>320</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>309</v>
+        <v>321</v>
       </c>
       <c r="D13" s="15" t="s">
         <v>6</v>
@@ -4291,13 +4367,13 @@
         <v>22</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>292</v>
+        <v>304</v>
       </c>
       <c r="H13" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>310</v>
+        <v>322</v>
       </c>
       <c r="J13" s="13" t="s">
         <v>45</v>
@@ -4308,13 +4384,13 @@
     </row>
     <row r="14" ht="75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>312</v>
+        <v>324</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>313</v>
+        <v>325</v>
       </c>
       <c r="D14" s="14" t="s">
         <v>7</v>
@@ -4323,33 +4399,33 @@
         <v>40</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>314</v>
+        <v>326</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>315</v>
+        <v>327</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>316</v>
+        <v>328</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
       <c r="J14" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>318</v>
+        <v>330</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>319</v>
+        <v>331</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
       <c r="D15" s="14" t="s">
         <v>7</v>
@@ -4361,13 +4437,13 @@
         <v>22</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>322</v>
+        <v>334</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>323</v>
+        <v>335</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>324</v>
+        <v>336</v>
       </c>
       <c r="J15" s="13" t="s">
         <v>45</v>
@@ -4378,13 +4454,13 @@
     </row>
     <row r="16" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>325</v>
+        <v>337</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>326</v>
+        <v>338</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="D16" s="12" t="s">
         <v>5</v>
@@ -4396,13 +4472,13 @@
         <v>22</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="H16" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
       <c r="J16" s="13" t="s">
         <v>45</v>
@@ -4413,13 +4489,13 @@
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>330</v>
+        <v>342</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>326</v>
+        <v>338</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>331</v>
+        <v>343</v>
       </c>
       <c r="D17" s="12" t="s">
         <v>5</v>
@@ -4431,30 +4507,30 @@
         <v>22</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="H17" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="J17" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K17" s="11" t="s">
-        <v>334</v>
+        <v>346</v>
       </c>
     </row>
     <row r="18" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>335</v>
+        <v>347</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>336</v>
+        <v>348</v>
       </c>
       <c r="D18" s="12" t="s">
         <v>5</v>
@@ -4466,13 +4542,13 @@
         <v>22</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>337</v>
+        <v>349</v>
       </c>
       <c r="H18" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>338</v>
+        <v>350</v>
       </c>
       <c r="J18" s="13" t="s">
         <v>45</v>
@@ -4483,13 +4559,13 @@
     </row>
     <row r="19" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>339</v>
+        <v>351</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>340</v>
+        <v>352</v>
       </c>
       <c r="D19" s="12" t="s">
         <v>5</v>
@@ -4501,13 +4577,13 @@
         <v>22</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>337</v>
+        <v>349</v>
       </c>
       <c r="H19" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>341</v>
+        <v>353</v>
       </c>
       <c r="J19" s="13" t="s">
         <v>45</v>
@@ -4518,13 +4594,13 @@
     </row>
     <row r="20" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>342</v>
+        <v>354</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>343</v>
+        <v>355</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>344</v>
+        <v>356</v>
       </c>
       <c r="D20" s="12" t="s">
         <v>5</v>
@@ -4533,33 +4609,33 @@
         <v>40</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>345</v>
+        <v>357</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="H20" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>347</v>
+        <v>359</v>
       </c>
       <c r="J20" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K20" s="11" t="s">
-        <v>348</v>
+        <v>360</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>349</v>
+        <v>361</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>343</v>
+        <v>355</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>350</v>
+        <v>362</v>
       </c>
       <c r="D21" s="14" t="s">
         <v>7</v>
@@ -4568,16 +4644,16 @@
         <v>104</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>351</v>
+        <v>363</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>352</v>
+        <v>364</v>
       </c>
       <c r="H21" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>353</v>
+        <v>365</v>
       </c>
       <c r="J21" s="13" t="s">
         <v>45</v>
@@ -4588,13 +4664,13 @@
     </row>
     <row r="22" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>354</v>
+        <v>366</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>355</v>
+        <v>367</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>356</v>
+        <v>368</v>
       </c>
       <c r="D22" s="12" t="s">
         <v>5</v>
@@ -4603,33 +4679,33 @@
         <v>40</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>357</v>
+        <v>369</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>337</v>
+        <v>349</v>
       </c>
       <c r="H22" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>358</v>
+        <v>370</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K22" s="11" t="s">
-        <v>359</v>
+        <v>371</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>360</v>
+        <v>372</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>355</v>
+        <v>367</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>361</v>
+        <v>373</v>
       </c>
       <c r="D23" s="15" t="s">
         <v>6</v>
@@ -4638,33 +4714,33 @@
         <v>104</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>362</v>
+        <v>374</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>337</v>
+        <v>349</v>
       </c>
       <c r="H23" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>363</v>
+        <v>375</v>
       </c>
       <c r="J23" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K23" s="11" t="s">
-        <v>364</v>
+        <v>376</v>
       </c>
     </row>
     <row r="24" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>365</v>
+        <v>377</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>366</v>
+        <v>378</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>367</v>
+        <v>379</v>
       </c>
       <c r="D24" s="15" t="s">
         <v>6</v>
@@ -4676,30 +4752,30 @@
         <v>22</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>352</v>
+        <v>364</v>
       </c>
       <c r="H24" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>368</v>
+        <v>380</v>
       </c>
       <c r="J24" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K24" s="11" t="s">
-        <v>369</v>
+        <v>381</v>
       </c>
     </row>
     <row r="25" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
-        <v>370</v>
+        <v>382</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>366</v>
+        <v>378</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="D25" s="15" t="s">
         <v>6</v>
@@ -4708,33 +4784,33 @@
         <v>83</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>372</v>
+        <v>384</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>352</v>
+        <v>364</v>
       </c>
       <c r="H25" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>373</v>
+        <v>385</v>
       </c>
       <c r="J25" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K25" s="11" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>375</v>
+        <v>387</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>377</v>
+        <v>389</v>
       </c>
       <c r="D26" s="12" t="s">
         <v>5</v>
@@ -4746,13 +4822,13 @@
         <v>22</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>378</v>
+        <v>390</v>
       </c>
       <c r="H26" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>379</v>
+        <v>391</v>
       </c>
       <c r="J26" s="13" t="s">
         <v>45</v>
@@ -4763,13 +4839,13 @@
     </row>
     <row r="27" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
-        <v>380</v>
+        <v>392</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>381</v>
+        <v>393</v>
       </c>
       <c r="D27" s="12" t="s">
         <v>5</v>
@@ -4778,22 +4854,22 @@
         <v>83</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>382</v>
+        <v>394</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
       <c r="H27" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>383</v>
+        <v>395</v>
       </c>
       <c r="J27" s="13" t="s">
         <v>45</v>
       </c>
       <c r="K27" s="11" t="s">
-        <v>384</v>
+        <v>396</v>
       </c>
     </row>
   </sheetData>
@@ -4820,35 +4896,35 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -4856,54 +4932,54 @@
         <v>11</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
     </row>
   </sheetData>
@@ -4914,7 +4990,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -4931,7 +5007,7 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>385</v>
+        <v>397</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -4946,7 +5022,7 @@
     </row>
     <row r="2" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>386</v>
+        <v>398</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -4961,7 +5037,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>387</v>
+        <v>399</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -5011,13 +5087,13 @@
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>388</v>
+        <v>400</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>130</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>389</v>
+        <v>401</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>6</v>
@@ -5026,33 +5102,33 @@
         <v>40</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>390</v>
+        <v>402</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>391</v>
+        <v>403</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>392</v>
+        <v>404</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>393</v>
+        <v>142</v>
       </c>
       <c r="K5" s="11" t="s">
-        <v>394</v>
+        <v>405</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>395</v>
+        <v>406</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>130</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>396</v>
+        <v>407</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>6</v>
@@ -5061,33 +5137,33 @@
         <v>83</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>397</v>
+        <v>408</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>398</v>
+        <v>409</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>399</v>
+        <v>410</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>400</v>
+        <v>411</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>393</v>
+        <v>142</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>401</v>
+        <v>412</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>402</v>
+        <v>413</v>
       </c>
       <c r="B7" s="11" t="s">
         <v>130</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>7</v>
@@ -5096,33 +5172,33 @@
         <v>104</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>404</v>
+        <v>415</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>391</v>
+        <v>403</v>
       </c>
       <c r="H7" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>405</v>
+        <v>416</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>393</v>
+        <v>142</v>
       </c>
       <c r="K7" s="11" t="s">
-        <v>406</v>
+        <v>417</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>407</v>
+        <v>418</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>130</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>408</v>
+        <v>419</v>
       </c>
       <c r="D8" s="15" t="s">
         <v>6</v>
@@ -5131,173 +5207,173 @@
         <v>40</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>397</v>
+        <v>408</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>409</v>
+        <v>420</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>410</v>
+        <v>421</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>411</v>
+        <v>422</v>
       </c>
       <c r="J8" s="13" t="s">
-        <v>393</v>
+        <v>142</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>401</v>
+        <v>412</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>412</v>
+        <v>423</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>413</v>
+        <v>130</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>414</v>
+        <v>424</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>6</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>40</v>
+        <v>104</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>415</v>
+        <v>408</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>416</v>
+        <v>425</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>22</v>
+        <v>426</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>417</v>
+        <v>427</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>393</v>
+        <v>142</v>
       </c>
       <c r="K9" s="11" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>419</v>
+        <v>428</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>38</v>
+        <v>429</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>420</v>
+        <v>430</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E10" s="11" t="s">
         <v>40</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>421</v>
+        <v>431</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>422</v>
+        <v>432</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>423</v>
+        <v>22</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>424</v>
+        <v>433</v>
       </c>
       <c r="J10" s="13" t="s">
-        <v>393</v>
+        <v>142</v>
       </c>
       <c r="K10" s="11" t="s">
-        <v>425</v>
+        <v>434</v>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>426</v>
+        <v>435</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>38</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>153</v>
+        <v>436</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E11" s="11" t="s">
         <v>40</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>154</v>
+        <v>437</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>427</v>
+        <v>438</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>22</v>
+        <v>439</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>428</v>
+        <v>440</v>
       </c>
       <c r="J11" s="13" t="s">
-        <v>429</v>
+        <v>142</v>
       </c>
       <c r="K11" s="11" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>431</v>
+        <v>442</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>432</v>
+        <v>443</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E12" s="11" t="s">
         <v>40</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>50</v>
+        <v>444</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>433</v>
+        <v>445</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>22</v>
+        <v>446</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>434</v>
+        <v>447</v>
       </c>
       <c r="J12" s="13" t="s">
-        <v>393</v>
+        <v>142</v>
       </c>
       <c r="K12" s="11" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="13" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>436</v>
+        <v>449</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>437</v>
+        <v>48</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>438</v>
+        <v>450</v>
       </c>
       <c r="D13" s="15" t="s">
         <v>5</v>
@@ -5306,208 +5382,208 @@
         <v>40</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>439</v>
+        <v>50</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>440</v>
+        <v>451</v>
       </c>
       <c r="H13" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="J13" s="13" t="s">
-        <v>393</v>
+        <v>142</v>
       </c>
       <c r="K13" s="11" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
-        <v>443</v>
+        <v>454</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>437</v>
+        <v>455</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>444</v>
+        <v>456</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>83</v>
+        <v>40</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>445</v>
+        <v>457</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>446</v>
+        <v>458</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>447</v>
+        <v>459</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>448</v>
+        <v>460</v>
       </c>
       <c r="J14" s="13" t="s">
-        <v>393</v>
+        <v>142</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>449</v>
+        <v>462</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>437</v>
+        <v>455</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>450</v>
+        <v>463</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>83</v>
+        <v>40</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>451</v>
+        <v>464</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>446</v>
+        <v>465</v>
       </c>
       <c r="H15" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>452</v>
+        <v>466</v>
       </c>
       <c r="J15" s="13" t="s">
-        <v>393</v>
+        <v>142</v>
       </c>
       <c r="K15" s="11" t="s">
-        <v>453</v>
+        <v>467</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
-        <v>454</v>
+        <v>468</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>48</v>
+        <v>455</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>455</v>
+        <v>469</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>40</v>
+        <v>83</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>456</v>
+        <v>470</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>457</v>
+        <v>471</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>22</v>
+        <v>472</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>458</v>
+        <v>473</v>
       </c>
       <c r="J16" s="13" t="s">
-        <v>393</v>
+        <v>142</v>
       </c>
       <c r="K16" s="11" t="s">
-        <v>22</v>
+        <v>472</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>459</v>
+        <v>474</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>460</v>
+        <v>455</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>461</v>
+        <v>475</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>40</v>
+        <v>83</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>462</v>
+        <v>476</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>463</v>
+        <v>471</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>464</v>
+        <v>22</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>465</v>
+        <v>477</v>
       </c>
       <c r="J17" s="13" t="s">
-        <v>393</v>
+        <v>142</v>
       </c>
       <c r="K17" s="11" t="s">
-        <v>22</v>
+        <v>478</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>466</v>
+        <v>479</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>460</v>
+        <v>48</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>467</v>
+        <v>480</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>83</v>
+        <v>40</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>22</v>
+        <v>481</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>468</v>
+        <v>482</v>
       </c>
       <c r="H18" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>469</v>
+        <v>483</v>
       </c>
       <c r="J18" s="13" t="s">
-        <v>429</v>
+        <v>142</v>
       </c>
       <c r="K18" s="11" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="19" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>471</v>
+        <v>484</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>472</v>
+        <v>485</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>473</v>
+        <v>486</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>5</v>
@@ -5516,68 +5592,68 @@
         <v>40</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>474</v>
+        <v>487</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>476</v>
+        <v>489</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>477</v>
+        <v>490</v>
       </c>
       <c r="J19" s="13" t="s">
-        <v>393</v>
+        <v>142</v>
       </c>
       <c r="K19" s="11" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="20" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>472</v>
+        <v>485</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>479</v>
+        <v>492</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>6</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>40</v>
+        <v>83</v>
       </c>
       <c r="F20" s="11" t="s">
         <v>22</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>480</v>
+        <v>493</v>
       </c>
       <c r="H20" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>481</v>
+        <v>494</v>
       </c>
       <c r="J20" s="13" t="s">
-        <v>429</v>
+        <v>495</v>
       </c>
       <c r="K20" s="11" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="21" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>483</v>
+        <v>497</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>484</v>
+        <v>498</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>485</v>
+        <v>499</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>5</v>
@@ -5586,33 +5662,33 @@
         <v>40</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>487</v>
+        <v>501</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>22</v>
+        <v>502</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>488</v>
+        <v>503</v>
       </c>
       <c r="J21" s="13" t="s">
-        <v>393</v>
+        <v>142</v>
       </c>
       <c r="K21" s="11" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>490</v>
+        <v>504</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>484</v>
+        <v>498</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>491</v>
+        <v>505</v>
       </c>
       <c r="D22" s="15" t="s">
         <v>6</v>
@@ -5624,138 +5700,138 @@
         <v>22</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>492</v>
+        <v>506</v>
       </c>
       <c r="H22" s="11" t="s">
-        <v>22</v>
+        <v>507</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>493</v>
+        <v>508</v>
       </c>
       <c r="J22" s="13" t="s">
-        <v>429</v>
+        <v>142</v>
       </c>
       <c r="K22" s="11" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="23" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>495</v>
+        <v>510</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>366</v>
+        <v>511</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>496</v>
+        <v>512</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E23" s="11" t="s">
         <v>40</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>22</v>
+        <v>513</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>497</v>
+        <v>514</v>
       </c>
       <c r="H23" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>498</v>
+        <v>515</v>
       </c>
       <c r="J23" s="13" t="s">
-        <v>429</v>
+        <v>142</v>
       </c>
       <c r="K23" s="11" t="s">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="24" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>500</v>
+        <v>517</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>366</v>
+        <v>511</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>501</v>
+        <v>518</v>
       </c>
       <c r="D24" s="15" t="s">
         <v>6</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>83</v>
+        <v>40</v>
       </c>
       <c r="F24" s="11" t="s">
         <v>22</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>502</v>
+        <v>519</v>
       </c>
       <c r="H24" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>503</v>
+        <v>520</v>
       </c>
       <c r="J24" s="13" t="s">
-        <v>429</v>
+        <v>495</v>
       </c>
       <c r="K24" s="11" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="25" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>506</v>
+        <v>378</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>507</v>
+        <v>523</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E25" s="11" t="s">
         <v>40</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>508</v>
+        <v>22</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>509</v>
+        <v>524</v>
       </c>
       <c r="H25" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>510</v>
+        <v>525</v>
       </c>
       <c r="J25" s="13" t="s">
-        <v>393</v>
+        <v>495</v>
       </c>
       <c r="K25" s="11" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="26" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>512</v>
+        <v>527</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>210</v>
+        <v>378</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>513</v>
+        <v>528</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>83</v>
@@ -5764,334 +5840,229 @@
         <v>22</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>514</v>
+        <v>529</v>
       </c>
       <c r="H26" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>515</v>
+        <v>530</v>
       </c>
       <c r="J26" s="13" t="s">
-        <v>393</v>
+        <v>495</v>
       </c>
       <c r="K26" s="11" t="s">
-        <v>22</v>
+        <v>531</v>
       </c>
     </row>
     <row r="27" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
-        <v>516</v>
+        <v>532</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>210</v>
+        <v>533</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>517</v>
+        <v>534</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>83</v>
+        <v>40</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>518</v>
+        <v>535</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>519</v>
+        <v>536</v>
       </c>
       <c r="H27" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>520</v>
+        <v>537</v>
       </c>
       <c r="J27" s="13" t="s">
-        <v>393</v>
+        <v>142</v>
       </c>
       <c r="K27" s="11" t="s">
-        <v>521</v>
+        <v>538</v>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
-        <v>522</v>
+        <v>539</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>123</v>
+        <v>223</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>523</v>
+        <v>540</v>
       </c>
       <c r="D28" s="15" t="s">
         <v>5</v>
       </c>
       <c r="E28" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F28" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="G28" s="11" t="s">
+        <v>541</v>
+      </c>
+      <c r="H28" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I28" s="11" t="s">
+        <v>542</v>
+      </c>
+      <c r="J28" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="K28" s="11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="29" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
+        <v>543</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>223</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>544</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E29" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" s="11" t="s">
+        <v>545</v>
+      </c>
+      <c r="G29" s="11" t="s">
+        <v>546</v>
+      </c>
+      <c r="H29" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I29" s="11" t="s">
+        <v>547</v>
+      </c>
+      <c r="J29" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="K29" s="11" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="30" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="11" t="s">
+        <v>549</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>550</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>551</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E30" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F30" s="11" t="s">
+        <v>552</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>553</v>
+      </c>
+      <c r="H30" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I30" s="11" t="s">
+        <v>554</v>
+      </c>
+      <c r="J30" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="K30" s="11" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="31" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="11" t="s">
+        <v>556</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>557</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>558</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E31" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="F28" s="11" t="s">
-        <v>357</v>
-      </c>
-      <c r="G28" s="11" t="s">
-        <v>524</v>
-      </c>
-      <c r="H28" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="I28" s="11" t="s">
-        <v>525</v>
-      </c>
-      <c r="J28" s="13" t="s">
-        <v>393</v>
-      </c>
-      <c r="K28" s="11" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A29" s="11" t="s">
-        <v>527</v>
-      </c>
-      <c r="B29" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>528</v>
-      </c>
-      <c r="D29" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="E29" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="F29" s="11" t="s">
-        <v>529</v>
-      </c>
-      <c r="G29" s="11" t="s">
-        <v>530</v>
-      </c>
-      <c r="H29" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="I29" s="11" t="s">
-        <v>531</v>
-      </c>
-      <c r="J29" s="13" t="s">
-        <v>429</v>
-      </c>
-      <c r="K29" s="11" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="30" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" s="11" t="s">
-        <v>533</v>
-      </c>
-      <c r="B30" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>534</v>
-      </c>
-      <c r="D30" s="15" t="s">
+      <c r="F31" s="11" t="s">
+        <v>559</v>
+      </c>
+      <c r="G31" s="11" t="s">
+        <v>560</v>
+      </c>
+      <c r="H31" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I31" s="11" t="s">
+        <v>561</v>
+      </c>
+      <c r="J31" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="K31" s="11" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="11" t="s">
+        <v>563</v>
+      </c>
+      <c r="B32" s="11" t="s">
+        <v>557</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>564</v>
+      </c>
+      <c r="D32" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="E30" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="F30" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="G30" s="11" t="s">
-        <v>535</v>
-      </c>
-      <c r="H30" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="I30" s="11" t="s">
-        <v>536</v>
-      </c>
-      <c r="J30" s="13" t="s">
-        <v>429</v>
-      </c>
-      <c r="K30" s="11" t="s">
-        <v>537</v>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A31" s="11" t="s">
-        <v>538</v>
-      </c>
-      <c r="B31" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="C31" s="11" t="s">
-        <v>539</v>
-      </c>
-      <c r="D31" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="E31" s="11" t="s">
+      <c r="E32" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="F31" s="11" t="s">
-        <v>508</v>
-      </c>
-      <c r="G31" s="11" t="s">
-        <v>540</v>
-      </c>
-      <c r="H31" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="I31" s="11" t="s">
-        <v>541</v>
-      </c>
-      <c r="J31" s="13" t="s">
-        <v>429</v>
-      </c>
-      <c r="K31" s="11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="32" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" s="11" t="s">
-        <v>542</v>
-      </c>
-      <c r="B32" s="11" t="s">
-        <v>543</v>
-      </c>
-      <c r="C32" s="11" t="s">
-        <v>544</v>
-      </c>
-      <c r="D32" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="E32" s="11" t="s">
-        <v>83</v>
-      </c>
       <c r="F32" s="11" t="s">
-        <v>545</v>
+        <v>22</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>546</v>
+        <v>565</v>
       </c>
       <c r="H32" s="11" t="s">
-        <v>22</v>
+        <v>566</v>
       </c>
       <c r="I32" s="11" t="s">
-        <v>547</v>
+        <v>567</v>
       </c>
       <c r="J32" s="13" t="s">
-        <v>393</v>
+        <v>142</v>
       </c>
       <c r="K32" s="11" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="33" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" s="11" t="s">
-        <v>549</v>
-      </c>
-      <c r="B33" s="11" t="s">
-        <v>550</v>
-      </c>
-      <c r="C33" s="11" t="s">
-        <v>551</v>
-      </c>
-      <c r="D33" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="E33" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="F33" s="11" t="s">
-        <v>552</v>
-      </c>
-      <c r="G33" s="11" t="s">
-        <v>553</v>
-      </c>
-      <c r="H33" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="I33" s="11" t="s">
-        <v>554</v>
-      </c>
-      <c r="J33" s="13" t="s">
-        <v>393</v>
-      </c>
-      <c r="K33" s="11" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="34" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A34" s="11" t="s">
-        <v>556</v>
-      </c>
-      <c r="B34" s="11" t="s">
-        <v>550</v>
-      </c>
-      <c r="C34" s="11" t="s">
-        <v>557</v>
-      </c>
-      <c r="D34" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E34" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="F34" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="G34" s="11" t="s">
-        <v>558</v>
-      </c>
-      <c r="H34" s="11" t="s">
-        <v>559</v>
-      </c>
-      <c r="I34" s="11" t="s">
-        <v>560</v>
-      </c>
-      <c r="J34" s="13" t="s">
-        <v>393</v>
-      </c>
-      <c r="K34" s="11" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="35" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" s="11" t="s">
-        <v>562</v>
-      </c>
-      <c r="B35" s="11" t="s">
-        <v>376</v>
-      </c>
-      <c r="C35" s="11" t="s">
-        <v>563</v>
-      </c>
-      <c r="D35" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="E35" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="F35" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="G35" s="11" t="s">
-        <v>564</v>
-      </c>
-      <c r="H35" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="I35" s="11" t="s">
-        <v>565</v>
-      </c>
-      <c r="J35" s="13" t="s">
-        <v>393</v>
-      </c>
-      <c r="K35" s="11" t="s">
-        <v>22</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -6102,6 +6073,6 @@
     <mergeCell ref="A3:K3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Confluence page; clarify CI secrets; drop PDI cases not yet run
- docs/Confluence.md: team-facing overview (what each automation does,
  the PDI process and pass/fail rule, how to run, CI setup, coverage,
  troubleshooting), in plain Markdown that Confluence imports cleanly.
- README: exact value for each GitHub Actions secret, which are required,
  and that no variables are needed.
- Test cases: remove the 4 PDI cases that haven't happened in a real run
  and the matching coverage-gap row; PDI now 24 cases, workbook 83/83.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Test Cases/DMS_Automation_Test_Cases.xlsx
+++ b/Test Cases/DMS_Automation_Test_Cases.xlsx
@@ -16,12 +16,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="591">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="567">
   <si>
     <t>River DMS - E2E Automation Test Cases</t>
   </si>
   <si>
-    <t>Enquiry List, GSTR and MIS test cases executed on 25-Sep-2026; PDI Vehicle Details and ENQ-16/17 on 28-Sep-2026 — all against the live DMS (Microsoft Edge and Google Chrome). "Not run yet" = handled in code, not yet seen in a live run.</t>
+    <t xml:space="preserve">Enquiry List, GSTR and MIS test cases executed on 25-Sep-2026; PDI Vehicle Details and ENQ-16/17 on 28-Sep-2026 — all against the live DMS (Microsoft Edge and Google Chrome). </t>
   </si>
   <si>
     <t>Sheet</t>
@@ -1514,222 +1514,159 @@
     <t>PDI-16</t>
   </si>
   <si>
-    <t>Show loads a different vehicle / nothing</t>
-  </si>
-  <si>
-    <t>Show a chassis the DMS can't find</t>
-  </si>
-  <si>
-    <t>Skipped: "Show did not load this vehicle"; nothing saved; test red</t>
-  </si>
-  <si>
-    <t>Not run yet</t>
-  </si>
-  <si>
-    <t>Handled in code; no such chassis met yet</t>
+    <t>VIN lookup</t>
+  </si>
+  <si>
+    <t>Fill details from the VIN Details sheet</t>
+  </si>
+  <si>
+    <t>resources/VIN Details (1).xlsx</t>
+  </si>
+  <si>
+    <t>Find chassis in col A; col C -&gt; EngineNo, col B -&gt; BatteryDetails, col D -&gt; VehicleChargerNo; EditChassisReason = "Details updated"</t>
+  </si>
+  <si>
+    <t>VIN Details (1).xlsx (29,814 VINs)</t>
+  </si>
+  <si>
+    <t>All four fields filled with the sheet's values</t>
   </si>
   <si>
     <t>PDI-17</t>
   </si>
   <si>
-    <t>VIN lookup</t>
-  </si>
-  <si>
-    <t>Fill details from the VIN Details sheet</t>
-  </si>
-  <si>
-    <t>resources/VIN Details (1).xlsx</t>
-  </si>
-  <si>
-    <t>Find chassis in col A; col C -&gt; EngineNo, col B -&gt; BatteryDetails, col D -&gt; VehicleChargerNo; EditChassisReason = "Details updated"</t>
-  </si>
-  <si>
-    <t>VIN Details (1).xlsx (29,814 VINs)</t>
-  </si>
-  <si>
-    <t>All four fields filled with the sheet's values</t>
+    <t>Chassis not in the VIN Details sheet</t>
+  </si>
+  <si>
+    <t>Run with a chassis missing from the sheet (dry run)</t>
+  </si>
+  <si>
+    <t>Copy of the VIN sheet without P7BAABXX1JT059691</t>
+  </si>
+  <si>
+    <t>Skipped and listed as "Not in VIN Details sheet"; other chassis continue; test red</t>
+  </si>
+  <si>
+    <t>D71001: P7BAABXX1JT059691 skipped and listed; run red</t>
   </si>
   <si>
     <t>PDI-18</t>
   </si>
   <si>
-    <t>Chassis not in the VIN Details sheet</t>
-  </si>
-  <si>
-    <t>Run with a chassis missing from the sheet (dry run)</t>
-  </si>
-  <si>
-    <t>Copy of the VIN sheet without P7BAABXX1JT059691</t>
-  </si>
-  <si>
-    <t>Skipped and listed as "Not in VIN Details sheet"; other chassis continue; test red</t>
-  </si>
-  <si>
-    <t>D71001: P7BAABXX1JT059691 skipped and listed; run red</t>
+    <t>Save</t>
+  </si>
+  <si>
+    <t>Save and confirm the DMS kept the values</t>
+  </si>
+  <si>
+    <t>Form filled</t>
+  </si>
+  <si>
+    <t>Click Save (ctl00_cpMain_cmdSave), Show again, compare Engine / Battery / Charger</t>
+  </si>
+  <si>
+    <t>Status "Updated"; chassis number logged</t>
+  </si>
+  <si>
+    <t>160 chassis updated across 12 dealers on 28-Sep</t>
   </si>
   <si>
     <t>PDI-19</t>
   </si>
   <si>
-    <t>Save</t>
-  </si>
-  <si>
-    <t>Save and confirm the DMS kept the values</t>
-  </si>
-  <si>
-    <t>Form filled</t>
-  </si>
-  <si>
-    <t>Click Save (ctl00_cpMain_cmdSave), Show again, compare Engine / Battery / Charger</t>
-  </si>
-  <si>
-    <t>Status "Updated"; chassis number logged</t>
-  </si>
-  <si>
-    <t>160 chassis updated across 12 dealers on 28-Sep</t>
+    <t>Dry run</t>
+  </si>
+  <si>
+    <t>Fill the form without saving</t>
+  </si>
+  <si>
+    <t>PDI_DRY_RUN=1</t>
+  </si>
+  <si>
+    <t>npm run test:pdi:dry</t>
+  </si>
+  <si>
+    <t>Form filled for every blank chassis, Save never clicked</t>
+  </si>
+  <si>
+    <t>D71001: 10 filled (morning run); 10 of 11 filled + 1 not in VIN sheet (negative test); nothing saved</t>
   </si>
   <si>
     <t>PDI-20</t>
   </si>
   <si>
-    <t>Save clicked but the values were not kept</t>
-  </si>
-  <si>
-    <t>DMS rejects or ignores the change</t>
-  </si>
-  <si>
-    <t>"Save clicked but values not kept"; test red</t>
-  </si>
-  <si>
-    <t>Handled in code; not seen yet</t>
+    <t>Results Excel with a Dealers sheet</t>
+  </si>
+  <si>
+    <t>Run ends</t>
+  </si>
+  <si>
+    <t>Output/PDI_BlankChassis_&lt;time&gt;.xlsx: one row per chassis + every dealer checked</t>
   </si>
   <si>
     <t>PDI-21</t>
   </si>
   <si>
-    <t>Page times out mid-dealer: recover and retry</t>
-  </si>
-  <si>
-    <t>A click / fill times out (session dropped)</t>
-  </si>
-  <si>
-    <t>Log in again if the form is gone; retry that chassis once; continue with the rest</t>
-  </si>
-  <si>
-    <t>Added after 4 timeouts on 372002 (13:38 run). Those 4 were checked in the DMS afterwards: values match the VIN sheet</t>
+    <t>Results Excel is open in Excel (locked)</t>
+  </si>
+  <si>
+    <t>File locked</t>
+  </si>
+  <si>
+    <t>Run ends / daily report written</t>
+  </si>
+  <si>
+    <t>Saved beside it as &lt;name&gt;_&lt;timestamp&gt;.xlsx; run continues</t>
+  </si>
+  <si>
+    <t>Locked PDI_Daily_2026-09-28.xlsx: EBUSY -&gt; saved as _1790610722383.xlsx, run passed</t>
   </si>
   <si>
     <t>PDI-22</t>
   </si>
   <si>
-    <t>Page cannot be recovered</t>
-  </si>
-  <si>
-    <t>Recovery (re-login) also fails</t>
-  </si>
-  <si>
-    <t>Remaining chassis marked "Not attempted"; finished ones kept; next dealer still runs; test red</t>
-  </si>
-  <si>
-    <t>Handled in code</t>
+    <t>Dashboard</t>
+  </si>
+  <si>
+    <t>Interactive dashboard</t>
+  </si>
+  <si>
+    <t>PDI_Dashboard.html (saved in Output)</t>
+  </si>
+  <si>
+    <t>Open in a browser; click a dealer bar, outcome chips, search, sort columns, theme toggle, phone width</t>
+  </si>
+  <si>
+    <t>Table filters / sorts correctly; dark mode and phone layout work</t>
+  </si>
+  <si>
+    <t>Sample data: dealer + Error filter -&gt; "2 of 14"; no script errors; no sideways scroll at 390 px</t>
   </si>
   <si>
     <t>PDI-23</t>
   </si>
   <si>
-    <t>Dry run</t>
-  </si>
-  <si>
-    <t>Fill the form without saving</t>
-  </si>
-  <si>
-    <t>PDI_DRY_RUN=1</t>
-  </si>
-  <si>
-    <t>npm run test:pdi:dry</t>
-  </si>
-  <si>
-    <t>Form filled for every blank chassis, Save never clicked</t>
-  </si>
-  <si>
-    <t>D71001: 10 filled (morning run); 10 of 11 filled + 1 not in VIN sheet (negative test); nothing saved</t>
+    <t>Daily report</t>
+  </si>
+  <si>
+    <t>Combine the day's runs</t>
+  </si>
+  <si>
+    <t>Result files in Output</t>
+  </si>
+  <si>
+    <t>npm run report:pdi-daily</t>
+  </si>
+  <si>
+    <t>Latest result per chassis; dry runs left out; errors cleared by a later check shown as Updated</t>
+  </si>
+  <si>
+    <t>28-Sep: 5 runs -&gt; 160 chassis, 15 dealers; 372002's 4 timeouts shown as Updated</t>
   </si>
   <si>
     <t>PDI-24</t>
   </si>
   <si>
-    <t>Results Excel with a Dealers sheet</t>
-  </si>
-  <si>
-    <t>Run ends</t>
-  </si>
-  <si>
-    <t>Output/PDI_BlankChassis_&lt;time&gt;.xlsx: one row per chassis + every dealer checked</t>
-  </si>
-  <si>
-    <t>PDI-25</t>
-  </si>
-  <si>
-    <t>Results Excel is open in Excel (locked)</t>
-  </si>
-  <si>
-    <t>File locked</t>
-  </si>
-  <si>
-    <t>Run ends / daily report written</t>
-  </si>
-  <si>
-    <t>Saved beside it as &lt;name&gt;_&lt;timestamp&gt;.xlsx; run continues</t>
-  </si>
-  <si>
-    <t>Locked PDI_Daily_2026-09-28.xlsx: EBUSY -&gt; saved as _1790610722383.xlsx, run passed</t>
-  </si>
-  <si>
-    <t>PDI-26</t>
-  </si>
-  <si>
-    <t>Dashboard</t>
-  </si>
-  <si>
-    <t>Interactive dashboard</t>
-  </si>
-  <si>
-    <t>PDI_Dashboard.html (saved in Output)</t>
-  </si>
-  <si>
-    <t>Open in a browser; click a dealer bar, outcome chips, search, sort columns, theme toggle, phone width</t>
-  </si>
-  <si>
-    <t>Table filters / sorts correctly; dark mode and phone layout work</t>
-  </si>
-  <si>
-    <t>Sample data: dealer + Error filter -&gt; "2 of 14"; no script errors; no sideways scroll at 390 px</t>
-  </si>
-  <si>
-    <t>PDI-27</t>
-  </si>
-  <si>
-    <t>Daily report</t>
-  </si>
-  <si>
-    <t>Combine the day's runs</t>
-  </si>
-  <si>
-    <t>Result files in Output</t>
-  </si>
-  <si>
-    <t>npm run report:pdi-daily</t>
-  </si>
-  <si>
-    <t>Latest result per chassis; dry runs left out; errors cleared by a later check shown as Updated</t>
-  </si>
-  <si>
-    <t>28-Sep: 5 runs -&gt; 160 chassis, 15 dealers; 372002's 4 timeouts shown as Updated</t>
-  </si>
-  <si>
-    <t>PDI-28</t>
-  </si>
-  <si>
     <t>No runs on that day</t>
   </si>
   <si>
@@ -1791,15 +1728,6 @@
   </si>
   <si>
     <t>Fixed (28-Sep-2026): the spec sets "Top" to PDI_TOP (500) and clicks Show; warns if the list is full — see the "top 25" PDI case</t>
-  </si>
-  <si>
-    <t>tests/PDI.spec.ts — not yet run live</t>
-  </si>
-  <si>
-    <t>PDI-16, PDI-20, PDI-21, PDI-22 are handled in code but have not happened in a real run yet</t>
-  </si>
-  <si>
-    <t>Mark them Pass the first time each one is seen</t>
   </si>
   <si>
     <t>tests/PDI.spec.ts — fixed 10 s wait after Show</t>
@@ -2432,13 +2360,13 @@
         <v>20</v>
       </c>
       <c r="C8" s="5">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D8" s="5">
         <v>12</v>
       </c>
       <c r="E8" s="5">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F8" s="5">
         <v>4</v>
@@ -2458,13 +2386,13 @@
         <v>22</v>
       </c>
       <c r="C9" s="6">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D9" s="6">
         <v>48</v>
       </c>
       <c r="E9" s="6">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F9" s="6">
         <v>14</v>
@@ -4886,7 +4814,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
@@ -4896,35 +4824,35 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>568</v>
+        <v>547</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>569</v>
+        <v>548</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>570</v>
+        <v>549</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>571</v>
+        <v>550</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>572</v>
+        <v>551</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>573</v>
+        <v>552</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>574</v>
+        <v>553</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>575</v>
+        <v>554</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>576</v>
+        <v>555</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -4932,54 +4860,43 @@
         <v>11</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>577</v>
+        <v>556</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>578</v>
+        <v>557</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>579</v>
+        <v>558</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>580</v>
+        <v>559</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>581</v>
+        <v>560</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>582</v>
+        <v>561</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>583</v>
+        <v>562</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>584</v>
+        <v>563</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>585</v>
+        <v>564</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>586</v>
+        <v>565</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
-        <v>588</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>589</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>590</v>
+        <v>566</v>
       </c>
     </row>
   </sheetData>
@@ -4990,7 +4907,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -5610,120 +5527,120 @@
         <v>22</v>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
         <v>491</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>485</v>
+        <v>492</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>83</v>
+        <v>40</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>22</v>
+        <v>494</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="H20" s="11" t="s">
-        <v>22</v>
+        <v>496</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="J20" s="13" t="s">
-        <v>495</v>
+        <v>142</v>
       </c>
       <c r="K20" s="11" t="s">
-        <v>496</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>498</v>
+        <v>492</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>499</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E21" s="11" t="s">
         <v>40</v>
       </c>
       <c r="F21" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="G21" s="11" t="s">
         <v>500</v>
       </c>
-      <c r="G21" s="11" t="s">
+      <c r="H21" s="11" t="s">
         <v>501</v>
       </c>
-      <c r="H21" s="11" t="s">
+      <c r="I21" s="11" t="s">
         <v>502</v>
-      </c>
-      <c r="I21" s="11" t="s">
-        <v>503</v>
       </c>
       <c r="J21" s="13" t="s">
         <v>142</v>
       </c>
       <c r="K21" s="11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="22" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
         <v>504</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>498</v>
+        <v>505</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>40</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>22</v>
+        <v>507</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="H22" s="11" t="s">
-        <v>507</v>
+        <v>22</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="J22" s="13" t="s">
         <v>142</v>
       </c>
       <c r="K22" s="11" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="23" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="D23" s="15" t="s">
         <v>5</v>
@@ -5732,138 +5649,138 @@
         <v>40</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="H23" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="J23" s="13" t="s">
         <v>142</v>
       </c>
       <c r="K23" s="11" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>511</v>
+        <v>223</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>40</v>
+        <v>83</v>
       </c>
       <c r="F24" s="11" t="s">
         <v>22</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="H24" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I24" s="11" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="J24" s="13" t="s">
-        <v>495</v>
+        <v>142</v>
       </c>
       <c r="K24" s="11" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="25" ht="60" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
         <v>522</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>378</v>
+        <v>223</v>
       </c>
       <c r="C25" s="11" t="s">
         <v>523</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>40</v>
+        <v>83</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>22</v>
+        <v>524</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="H25" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="J25" s="13" t="s">
-        <v>495</v>
+        <v>142</v>
       </c>
       <c r="K25" s="11" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
     </row>
     <row r="26" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>378</v>
+        <v>529</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>83</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>22</v>
+        <v>531</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="H26" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="J26" s="13" t="s">
-        <v>495</v>
+        <v>142</v>
       </c>
       <c r="K26" s="11" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
     </row>
     <row r="27" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="D27" s="15" t="s">
         <v>5</v>
@@ -5872,196 +5789,56 @@
         <v>40</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="H27" s="11" t="s">
         <v>22</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="J27" s="13" t="s">
         <v>142</v>
       </c>
       <c r="K27" s="11" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>223</v>
+        <v>536</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>83</v>
+        <v>104</v>
       </c>
       <c r="F28" s="11" t="s">
         <v>22</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>22</v>
+        <v>545</v>
       </c>
       <c r="I28" s="11" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
       <c r="J28" s="13" t="s">
         <v>142</v>
       </c>
       <c r="K28" s="11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="29" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A29" s="11" t="s">
-        <v>543</v>
-      </c>
-      <c r="B29" s="11" t="s">
-        <v>223</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>544</v>
-      </c>
-      <c r="D29" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="E29" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="F29" s="11" t="s">
-        <v>545</v>
-      </c>
-      <c r="G29" s="11" t="s">
-        <v>546</v>
-      </c>
-      <c r="H29" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="I29" s="11" t="s">
-        <v>547</v>
-      </c>
-      <c r="J29" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="K29" s="11" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="30" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" s="11" t="s">
-        <v>549</v>
-      </c>
-      <c r="B30" s="11" t="s">
-        <v>550</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>551</v>
-      </c>
-      <c r="D30" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="E30" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="F30" s="11" t="s">
-        <v>552</v>
-      </c>
-      <c r="G30" s="11" t="s">
-        <v>553</v>
-      </c>
-      <c r="H30" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="I30" s="11" t="s">
-        <v>554</v>
-      </c>
-      <c r="J30" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="K30" s="11" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="31" ht="45" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A31" s="11" t="s">
-        <v>556</v>
-      </c>
-      <c r="B31" s="11" t="s">
-        <v>557</v>
-      </c>
-      <c r="C31" s="11" t="s">
-        <v>558</v>
-      </c>
-      <c r="D31" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="E31" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="F31" s="11" t="s">
-        <v>559</v>
-      </c>
-      <c r="G31" s="11" t="s">
-        <v>560</v>
-      </c>
-      <c r="H31" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="I31" s="11" t="s">
-        <v>561</v>
-      </c>
-      <c r="J31" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="K31" s="11" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" s="11" t="s">
-        <v>563</v>
-      </c>
-      <c r="B32" s="11" t="s">
-        <v>557</v>
-      </c>
-      <c r="C32" s="11" t="s">
-        <v>564</v>
-      </c>
-      <c r="D32" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E32" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="F32" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="G32" s="11" t="s">
-        <v>565</v>
-      </c>
-      <c r="H32" s="11" t="s">
-        <v>566</v>
-      </c>
-      <c r="I32" s="11" t="s">
-        <v>567</v>
-      </c>
-      <c r="J32" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="K32" s="11" t="s">
         <v>149</v>
       </c>
     </row>

</xml_diff>

<commit_message>
PDI: 3-day master, all-time tracking, Excel-only daily email
- PDI_Master.xlsx keeps the last 3 days (was 2) and opens on a new
  Tracking sheet: all-time chassis found / updated / no usable VIN data,
  plus one row per day with running totals.
- New Output/PDI_History.json (pdiHistory.ts) keeps every day for good;
  the 3-day clean-up never deletes it.
- New PDI_Master.html dashboard (saved locally): totals, day-wise chart,
  updated chassis per dealer per day, filterable chassis table.
- Daily email shows "till now" KPIs and a day-wise tracking table; only
  Excel files are attached (daily workbook + PDI_Master.xlsx).
- PDI_EMAIL_REVIEW=1 documented; generic Gmail reporter skips PDI runs.
- Test cases PDI-25..PDI-32, README and Confluence page updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Test Cases/DMS_Automation_Test_Cases.xlsx
+++ b/Test Cases/DMS_Automation_Test_Cases.xlsx
@@ -15,13 +15,26 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="H8" authorId="0">
+      <text/>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="567">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1103" uniqueCount="620">
   <si>
     <t>River DMS - E2E Automation Test Cases</t>
   </si>
   <si>
-    <t xml:space="preserve">Enquiry List, GSTR and MIS test cases executed on 25-Sep-2026; PDI Vehicle Details and ENQ-16/17 on 28-Sep-2026 — all against the live DMS (Microsoft Edge and Google Chrome). </t>
+    <t>Enquiry List, GSTR and MIS test cases executed on 25-Sep-2026; PDI Vehicle Details and ENQ-16/17 on 28-Sep-2026; PDI master, tracking and email cases (PDI-25 to PDI-32) on 01-Oct-2026 — all against the live DMS (Microsoft Edge and Google Chrome). PDI-29 / PDI-30 are pending the report owner's review of the email.</t>
   </si>
   <si>
     <t>Sheet</t>
@@ -1677,6 +1690,165 @@
   </si>
   <si>
     <t>Stops: "No PDI result files from 2020-01-01"</t>
+  </si>
+  <si>
+    <t>PDI-25</t>
+  </si>
+  <si>
+    <t>Master</t>
+  </si>
+  <si>
+    <t>PDI master keeps the last 3 days</t>
+  </si>
+  <si>
+    <t>PDI_Daily files for 29-Sep, 30-Sep and 01-Oct in Output</t>
+  </si>
+  <si>
+    <t>npm run report:pdi-daily (any rebuild of the daily report)</t>
+  </si>
+  <si>
+    <t>Output/PDI_Master.xlsx: Tracking sheet, then one sheet per day for the last 3 days (newest first); older PDI files deleted, GSTR/other outputs untouched</t>
+  </si>
+  <si>
+    <t>Pass (01-Oct-2026)</t>
+  </si>
+  <si>
+    <t>Sheets: Tracking, 2026-10-01 (90 chassis), 2026-09-30 (237), 2026-09-29 (371)</t>
+  </si>
+  <si>
+    <t>PDI-26</t>
+  </si>
+  <si>
+    <t>Build a past day's report without emailing</t>
+  </si>
+  <si>
+    <t>Run files for that day in Output/PDI runs</t>
+  </si>
+  <si>
+    <t>PDI_RUN=1 PDI_REPORT_DATE=2026-09-30 PDI_SEND_EMAIL=0 npx playwright test tests/PDIDailyReport.spec.ts</t>
+  </si>
+  <si>
+    <t>PDI_REPORT_DATE=2026-09-30, PDI_SEND_EMAIL=0</t>
+  </si>
+  <si>
+    <t>PDI_Daily_&lt;day&gt;.xlsx built from that day's runs and added to the master; no email sent</t>
+  </si>
+  <si>
+    <t>30-Sep: 3 runs -&gt; 237 chassis, 85 dealers; "PDI_SEND_EMAIL=0 — report email skipped"</t>
+  </si>
+  <si>
+    <t>PDI-27</t>
+  </si>
+  <si>
+    <t>Tracking</t>
+  </si>
+  <si>
+    <t>All-time totals and day-wise running totals</t>
+  </si>
+  <si>
+    <t>Output/PDI_History.json (filled by every daily rebuild)</t>
+  </si>
+  <si>
+    <t>Rebuild the daily report; open the Tracking sheet of PDI_Master.xlsx</t>
+  </si>
+  <si>
+    <t>29-Sep to 01-Oct history</t>
+  </si>
+  <si>
+    <t>KPIs: total chassis found, total updated, no usable VIN data (still open), errors (still open); one row per day with that day's counts and running totals</t>
+  </si>
+  <si>
+    <t>693 found / 679 updated / 14 no VIN / 0 errors; running totals found 371 -&gt; 607 -&gt; 693, updated 370 -&gt; 603 -&gt; 679</t>
+  </si>
+  <si>
+    <t>PDI-28</t>
+  </si>
+  <si>
+    <t>PDI master dashboard</t>
+  </si>
+  <si>
+    <t>Output/PDI_Master.html (saved in Output, not emailed)</t>
+  </si>
+  <si>
+    <t>Open in a browser: KPI tiles, day-wise bars (click a day to filter), dealer x day table, chassis table with filters/search/sort; theme toggle; phone width</t>
+  </si>
+  <si>
+    <t>All sections render and filter; dark mode and phone layout work</t>
+  </si>
+  <si>
+    <t>No script errors; no sideways scroll at 390 px; light and dark checked</t>
+  </si>
+  <si>
+    <t>PDI-29</t>
+  </si>
+  <si>
+    <t>"Till now" KPIs and day-wise tracking in the email body</t>
+  </si>
+  <si>
+    <t>PDI history present</t>
+  </si>
+  <si>
+    <t>PDI_RUN=1 PDI_EMAIL_REVIEW=1 PDI_FORCE_EMAIL=1 npx playwright test tests/PDIDailyReport.spec.ts</t>
+  </si>
+  <si>
+    <t>Email body shows total chassis found / updated / no usable VIN data (still open) since the first day, and a day-wise table (last 14 days) with running totals</t>
+  </si>
+  <si>
+    <t>Pending review</t>
+  </si>
+  <si>
+    <t>Review copy sent 01-Oct-2026 with 693 / 679 / 14; layout to be confirmed by the report owner</t>
+  </si>
+  <si>
+    <t>PDI-30</t>
+  </si>
+  <si>
+    <t>Only Excel files are attached</t>
+  </si>
+  <si>
+    <t>PDI_Master.xlsx in Output</t>
+  </si>
+  <si>
+    <t>Send the daily report</t>
+  </si>
+  <si>
+    <t>Attachments: PDI_Daily_&lt;day&gt;.xlsx and PDI_Master.xlsx; no HTML files</t>
+  </si>
+  <si>
+    <t>Review copy sent 01-Oct-2026; to be confirmed in the inbox</t>
+  </si>
+  <si>
+    <t>PDI-31</t>
+  </si>
+  <si>
+    <t>Review copy goes to the report owner only</t>
+  </si>
+  <si>
+    <t>Today's email already sent</t>
+  </si>
+  <si>
+    <t>PDI_EMAIL_REVIEW=1</t>
+  </si>
+  <si>
+    <t>Sent to GMAIL_TO only, subject starts [REVIEW], no CC; the day's "emailed" marker is not changed</t>
+  </si>
+  <si>
+    <t>"Report emailed to sunita@rideriver.com." (no cc); emailed_2026-10-01.txt still "sent 11:48"</t>
+  </si>
+  <si>
+    <t>PDI-32</t>
+  </si>
+  <si>
+    <t>Daily email is not sent twice</t>
+  </si>
+  <si>
+    <t>Run npm run report:pdi-daily again the same day</t>
+  </si>
+  <si>
+    <t>Report files rebuilt; email skipped with a message</t>
+  </si>
+  <si>
+    <t>"Today's PDI email already went out (sent 1/10/2026, 11:48:52 am) — not sending it again"</t>
   </si>
   <si>
     <t>Item</t>
@@ -1781,7 +1953,7 @@
       <name val="Consolas"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1818,6 +1990,11 @@
         <fgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1838,7 +2015,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1873,6 +2050,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2360,19 +2540,19 @@
         <v>20</v>
       </c>
       <c r="C8" s="5">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="D8" s="5">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E8" s="5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F8" s="5">
         <v>4</v>
       </c>
       <c r="G8" s="5">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>21</v>
@@ -2386,19 +2566,19 @@
         <v>22</v>
       </c>
       <c r="C9" s="6">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="D9" s="6">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="E9" s="6">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F9" s="6">
         <v>14</v>
       </c>
       <c r="G9" s="6">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>22</v>
@@ -2417,6 +2597,7 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <legacyDrawing r:id="rId6"/>
 </worksheet>
 </file>
 
@@ -4823,36 +5004,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
-        <v>547</v>
-      </c>
-      <c r="B1" s="16" t="s">
-        <v>548</v>
-      </c>
-      <c r="C1" s="16" t="s">
-        <v>549</v>
+      <c r="A1" s="17" t="s">
+        <v>600</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>601</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>602</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>550</v>
+        <v>603</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>551</v>
+        <v>604</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>552</v>
+        <v>605</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>553</v>
+        <v>606</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>554</v>
+        <v>607</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>555</v>
+        <v>608</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -4860,43 +5041,43 @@
         <v>11</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>556</v>
+        <v>609</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>557</v>
+        <v>610</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>558</v>
+        <v>611</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>559</v>
+        <v>612</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>560</v>
+        <v>613</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>561</v>
+        <v>614</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>562</v>
+        <v>615</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>563</v>
+        <v>616</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>564</v>
+        <v>617</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>565</v>
+        <v>618</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>566</v>
+        <v>619</v>
       </c>
     </row>
   </sheetData>
@@ -4907,7 +5088,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -5842,6 +6023,286 @@
         <v>149</v>
       </c>
     </row>
+    <row r="29" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
+        <v>547</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>548</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>549</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E29" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F29" s="11" t="s">
+        <v>550</v>
+      </c>
+      <c r="G29" s="11" t="s">
+        <v>551</v>
+      </c>
+      <c r="H29" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I29" s="11" t="s">
+        <v>552</v>
+      </c>
+      <c r="J29" s="13" t="s">
+        <v>553</v>
+      </c>
+      <c r="K29" s="11" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="11" t="s">
+        <v>555</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>536</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>556</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E30" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F30" s="11" t="s">
+        <v>557</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>558</v>
+      </c>
+      <c r="H30" s="11" t="s">
+        <v>559</v>
+      </c>
+      <c r="I30" s="11" t="s">
+        <v>560</v>
+      </c>
+      <c r="J30" s="13" t="s">
+        <v>553</v>
+      </c>
+      <c r="K30" s="11" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="11" t="s">
+        <v>562</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>563</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>564</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E31" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F31" s="11" t="s">
+        <v>565</v>
+      </c>
+      <c r="G31" s="11" t="s">
+        <v>566</v>
+      </c>
+      <c r="H31" s="11" t="s">
+        <v>567</v>
+      </c>
+      <c r="I31" s="11" t="s">
+        <v>568</v>
+      </c>
+      <c r="J31" s="13" t="s">
+        <v>553</v>
+      </c>
+      <c r="K31" s="11" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="11" t="s">
+        <v>570</v>
+      </c>
+      <c r="B32" s="11" t="s">
+        <v>529</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>571</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E32" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F32" s="11" t="s">
+        <v>572</v>
+      </c>
+      <c r="G32" s="11" t="s">
+        <v>573</v>
+      </c>
+      <c r="H32" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I32" s="11" t="s">
+        <v>574</v>
+      </c>
+      <c r="J32" s="13" t="s">
+        <v>553</v>
+      </c>
+      <c r="K32" s="11" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="11" t="s">
+        <v>576</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>367</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>577</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E33" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F33" s="11" t="s">
+        <v>578</v>
+      </c>
+      <c r="G33" s="11" t="s">
+        <v>579</v>
+      </c>
+      <c r="H33" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I33" s="11" t="s">
+        <v>580</v>
+      </c>
+      <c r="J33" s="16" t="s">
+        <v>581</v>
+      </c>
+      <c r="K33" s="11" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="11" t="s">
+        <v>583</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>367</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>584</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E34" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>585</v>
+      </c>
+      <c r="G34" s="11" t="s">
+        <v>586</v>
+      </c>
+      <c r="H34" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I34" s="11" t="s">
+        <v>587</v>
+      </c>
+      <c r="J34" s="16" t="s">
+        <v>581</v>
+      </c>
+      <c r="K34" s="11" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="11" t="s">
+        <v>589</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>367</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>590</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E35" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F35" s="11" t="s">
+        <v>591</v>
+      </c>
+      <c r="G35" s="11" t="s">
+        <v>579</v>
+      </c>
+      <c r="H35" s="11" t="s">
+        <v>592</v>
+      </c>
+      <c r="I35" s="11" t="s">
+        <v>593</v>
+      </c>
+      <c r="J35" s="13" t="s">
+        <v>553</v>
+      </c>
+      <c r="K35" s="11" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="11" t="s">
+        <v>595</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>367</v>
+      </c>
+      <c r="C36" s="11" t="s">
+        <v>596</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E36" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F36" s="11" t="s">
+        <v>591</v>
+      </c>
+      <c r="G36" s="11" t="s">
+        <v>597</v>
+      </c>
+      <c r="H36" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I36" s="11" t="s">
+        <v>598</v>
+      </c>
+      <c r="J36" s="13" t="s">
+        <v>553</v>
+      </c>
+      <c r="K36" s="11" t="s">
+        <v>599</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A4:K4"/>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Rebuild Product-wise Sales Invoice/Booking and the Enquiry summary
- Enquiry List spec again reads Product-wise Sales Details by Invoice and by
  Booking date in the same session, counts dealers, and builds the Enquiry /
  Invoice / Booking summary by date and dealer (removed on 01-Oct)
- Summary saved to Output/Enquiry_Summary_<from>_<to>.xlsx (By Date, By Dealer,
  By Date and Dealer); the per-day table goes in the run email
- Data checks on both sales reports; summary totals must match the reports
- Fixes from the old version: bookings already invoiced count on their booking
  date; dates sort by date, not as text
- Read dd-Mon-yyyy dates: the Enquiry List export changed to 07-Sep-2026
- Test cases: ENQ-08 to 13 pass on 08-Oct, ENQ-14 pending an emailed run,
  new ENQ-18 to 21

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Test Cases/DMS_Automation_Test_Cases.xlsx
+++ b/Test Cases/DMS_Automation_Test_Cases.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enquiry List" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GSTR Report" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MIS Report Check" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PDI Vehicle Details" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stage DMS Flow" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Gaps" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Enquiry List" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="GSTR Report" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="MIS Report Check" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="PDI Vehicle Details" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Stage DMS Flow" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Coverage Gaps" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Enquiry List'!$A$4:$K$4</definedName>
@@ -602,7 +602,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Enquiry List, GSTR and MIS test cases executed on 25-Sep-2026; PDI Vehicle Details and ENQ-16/17 on 28-Sep-2026; PDI master, tracking and email cases (PDI-25 to PDI-32) on 01-Oct-2026 — all against the live DMS (Microsoft Edge and Google Chrome). PDI-29 / PDI-30 are pending the report owner's review of the email. Stage DMS flow (STG-01 to STG-05) on 06-Oct-2026 against the stage DMS (Google Chrome).</t>
+          <t>Enquiry List, GSTR and MIS test cases executed on 25-Sep-2026; PDI Vehicle Details and ENQ-16/17 on 28-Sep-2026; PDI master, tracking and email cases (PDI-25 to PDI-32) on 01-Oct-2026 — all against the live DMS (Microsoft Edge and Google Chrome). PDI-29 / PDI-30 are pending the report owner's review of the email. Stage DMS flow (STG-01 to STG-05) on 06-Oct-2026 against the stage DMS (Google Chrome). Enquiry List rebuilt on 08-Oct-2026 (ENQ-05 to ENQ-21, Google Chrome); ENQ-14 is pending an emailed run.</t>
         </is>
       </c>
     </row>
@@ -660,19 +660,19 @@
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
@@ -816,19 +816,19 @@
       </c>
       <c r="B10" s="6" t="inlineStr"/>
       <c r="C10" s="6" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>22</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="H10" s="6" t="inlineStr"/>
     </row>
@@ -855,7 +855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1211,12 +1211,12 @@
       </c>
       <c r="J9" s="13" t="inlineStr">
         <is>
-          <t>Pass (25-Sep-2026)</t>
+          <t>Pass (08-Oct-2026)</t>
         </is>
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>20,113 enquiries</t>
+          <t>31,972 enquiries (07-Sep to 07-Oct-2026). Also covered by the data checks in ENQ-18</t>
         </is>
       </c>
     </row>
@@ -1266,12 +1266,12 @@
       </c>
       <c r="J10" s="13" t="inlineStr">
         <is>
-          <t>Pass (25-Sep-2026)</t>
+          <t>Pass (08-Oct-2026)</t>
         </is>
       </c>
       <c r="K10" s="11" t="inlineStr">
         <is>
-          <t>All three reports were over the limit: Enquiry 20,113, Invoice 3,171, Booking 4,709 rows - all read from the Excel download</t>
+          <t>All three reports over the limit: Enquiry 31,972, Invoice 5,112, Booking 7,649 rows</t>
         </is>
       </c>
     </row>
@@ -1308,23 +1308,23 @@
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>Read Dealer Code column by header name</t>
+          <t>Read Dealer Code from each report's rows (Dealer Code / DealerCode)</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr"/>
       <c r="I11" s="11" t="inlineStr">
         <is>
-          <t>Dealer code list and distinct dealer count logged</t>
+          <t>Row count and distinct dealer count logged per report</t>
         </is>
       </c>
       <c r="J11" s="13" t="inlineStr">
         <is>
-          <t>Pass (25-Sep-2026)</t>
+          <t>Pass (08-Oct-2026)</t>
         </is>
       </c>
       <c r="K11" s="11" t="inlineStr">
         <is>
-          <t>87 distinct dealers (Enquiry), 84 (Booking)</t>
+          <t>Enquiry 95, Invoice 86, Booking 92 distinct dealers. Rebuilt 08-Oct after removal on 01-Oct</t>
         </is>
       </c>
     </row>
@@ -1361,23 +1361,23 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Group rows; print table with Total row</t>
+          <t>Group by Date + Dealer Code (dates parsed, oldest first); add Total row</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr"/>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>Table printed; Total = record count</t>
+          <t>Grouped table with Total row; Total = record count</t>
         </is>
       </c>
       <c r="J12" s="13" t="inlineStr">
         <is>
-          <t>Pass (25-Sep-2026)</t>
+          <t>Pass (08-Oct-2026)</t>
         </is>
       </c>
       <c r="K12" s="11" t="inlineStr">
         <is>
-          <t>Total row = 20,113</t>
+          <t>Part of the combined summary (ENQ-13): Enquiry total 31,972 = record count</t>
         </is>
       </c>
     </row>
@@ -1431,12 +1431,12 @@
       </c>
       <c r="J13" s="13" t="inlineStr">
         <is>
-          <t>Pass (25-Sep-2026)</t>
+          <t>Pass (08-Oct-2026)</t>
         </is>
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>3,171 invoice rows</t>
+          <t>5,112 invoice rows, counted by distinct Booking No on Invoice Date</t>
         </is>
       </c>
     </row>
@@ -1484,12 +1484,12 @@
       </c>
       <c r="J14" s="13" t="inlineStr">
         <is>
-          <t>Pass (25-Sep-2026)</t>
+          <t>Pass (08-Oct-2026)</t>
         </is>
       </c>
       <c r="K14" s="11" t="inlineStr">
         <is>
-          <t>Google Chrome run: "Dealer codes: 3239 rows, 83 distinct dealers" for Invoice</t>
+          <t>Invoice: 5,112 rows from 86 dealers</t>
         </is>
       </c>
     </row>
@@ -1539,17 +1539,17 @@
       </c>
       <c r="I15" s="11" t="inlineStr">
         <is>
-          <t>Booking count &gt; 0; alert with count</t>
+          <t>Booking rows read (soft check: count &gt; 0); counted by distinct Booking No on Booking Date</t>
         </is>
       </c>
       <c r="J15" s="13" t="inlineStr">
         <is>
-          <t>Pass (25-Sep-2026)</t>
+          <t>Pass (08-Oct-2026)</t>
         </is>
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>4,709 booking rows</t>
+          <t>7,649 booking rows. Bookings already invoiced now count on their booking date, not the invoice date (bug in the 25-Sep version)</t>
         </is>
       </c>
     </row>
@@ -1592,17 +1592,17 @@
       <c r="H16" s="11" t="inlineStr"/>
       <c r="I16" s="11" t="inlineStr">
         <is>
-          <t>Combined table printed; combined-summary.csv attached to the test result</t>
+          <t>Output/Enquiry_Summary_&lt;from&gt;_&lt;to&gt;.xlsx with sheets By Date, By Dealer, By Date and Dealer, each with a Total row; per-day CSV attached to the test result</t>
         </is>
       </c>
       <c r="J16" s="13" t="inlineStr">
         <is>
-          <t>Pass (25-Sep-2026)</t>
+          <t>Pass (08-Oct-2026)</t>
         </is>
       </c>
       <c r="K16" s="11" t="inlineStr">
         <is>
-          <t>Totals 20,113 / 3,171 / 4,709; combined-summary.csv attached</t>
+          <t>2,560 date/dealer rows; totals 31,972 / 5,112 / 7,649</t>
         </is>
       </c>
     </row>
@@ -1645,17 +1645,17 @@
       <c r="H17" s="11" t="inlineStr"/>
       <c r="I17" s="11" t="inlineStr">
         <is>
-          <t>Gmail reporter emails the CSV as an HTML table</t>
+          <t>Gmail reporter pastes the per-day Enquiry / Invoice / Booking table (enquiry-invoice-booking-by-date.csv) into the email body. The date/dealer table is in the Excel file only (about 2,500 rows, which Gmail would clip)</t>
         </is>
       </c>
       <c r="J17" s="13" t="inlineStr">
         <is>
-          <t>Pass (25-Sep-2026)</t>
+          <t>Pending (08-Oct-2026)</t>
         </is>
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>Emailed to sunita@rideriver.com with 1 report pasted in the body</t>
+          <t>Rebuilt 08-Oct. The verification runs had email switched off; confirm on the next CI or local run</t>
         </is>
       </c>
     </row>
@@ -1819,6 +1819,218 @@
       <c r="K20" s="11" t="inlineStr">
         <is>
           <t>Exact message seen</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>ENQ-18</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Data check</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Enquiry List data checks</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>Enquiry rows read</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>Check columns, blanks and Created Date range</t>
+        </is>
+      </c>
+      <c r="H21" s="11" t="inlineStr"/>
+      <c r="I21" s="11" t="inlineStr">
+        <is>
+          <t>Key columns present; Dealer Code, Lead No and Created Date never blank; every Created Date inside the range. Soft, so the sales reports still run</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="inlineStr">
+        <is>
+          <t>Pass (08-Oct-2026)</t>
+        </is>
+      </c>
+      <c r="K21" s="11" t="inlineStr">
+        <is>
+          <t>No problems in 31,972 rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>ENQ-19</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Data check</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Invoice and Booking data checks</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>Both sales reports read</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>Check columns, Booking No / Dealer Code blanks and date range per report</t>
+        </is>
+      </c>
+      <c r="H22" s="11" t="inlineStr"/>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>Dealer Code, Dealer Name, Booking No and the date column present; no blank Booking No / Dealer Code; dates inside the range</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
+        <is>
+          <t>Pass (08-Oct-2026)</t>
+        </is>
+      </c>
+      <c r="K22" s="11" t="inlineStr">
+        <is>
+          <t>No problems in 5,112 + 7,649 rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>ENQ-20</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Summary totals match the reports</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>Summary built</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>Compare the Total row with each report</t>
+        </is>
+      </c>
+      <c r="H23" s="11" t="inlineStr"/>
+      <c r="I23" s="11" t="inlineStr">
+        <is>
+          <t>Enquiry total = enquiry rows; Invoice / Booking totals = distinct bookings per date and dealer</t>
+        </is>
+      </c>
+      <c r="J23" s="13" t="inlineStr">
+        <is>
+          <t>Pass (08-Oct-2026)</t>
+        </is>
+      </c>
+      <c r="K23" s="11" t="inlineStr">
+        <is>
+          <t>31,972 / 5,112 / 7,649 matched</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>ENQ-21</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Data check</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Enquiry Excel export uses dd-Mon-yyyy dates</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>Report over 1,000 rows</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>Run with the export that writes Created Date as 07-Sep-2026</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr"/>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>Dates read correctly; not reported as outside the range</t>
+        </is>
+      </c>
+      <c r="J24" s="13" t="inlineStr">
+        <is>
+          <t>Pass (08-Oct-2026)</t>
+        </is>
+      </c>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t>Found on 08-Oct: the export changed from 07-09-2026 to 07-Sep-2026. First run flagged all 31,972 rows; date reading fixed</t>
         </is>
       </c>
     </row>
@@ -6591,7 +6803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -6619,17 +6831,17 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Removed on 25-Sep (moved to "E2E DMS_removed_2026-09-25")</t>
+          <t>Finance Dashboard (legacy)</t>
         </is>
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>Finance Dashboard helpers (utils/appsScriptSheet.ts, utils/excelExport.ts, resources/apps-script), unused Spares page objects, old tests/MIS Report_Check.js, requirements.txt, specs/, resources/credentials.ts</t>
+          <t>tests/FinanaceDashboard.spec.ts, utils/appsScriptSheet.ts, utils/excelExport.ts and resources/apps-script are still in the project (an earlier note said they were removed). The spec has no assertions and runs under npm test</t>
         </is>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Nothing - kept outside the project only as a backup</t>
+          <t>Decide: delete them, or keep and add checks</t>
         </is>
       </c>
     </row>
@@ -6680,7 +6892,7 @@
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>Needs the repository owner: add the secrets under Settings &gt; Secrets and variables &gt; Actions, then run the workflow once (cannot be done from this PC — no GitHub CLI / secret values are private)</t>
+          <t>Secrets added 08-Oct-2026. The workflow first checks GitHub can reach the DMS and stops with a clear message if not</t>
         </is>
       </c>
     </row>
@@ -6697,7 +6909,7 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Fixed (28-Sep-2026): the spec sets "Top" to PDI_TOP (500) and clicks Show; warns if the list is full — see the "top 25" PDI case</t>
+          <t>Fixed: Top is set to the page's own "Displaying : N" count (PDI_TOP removed 08-Oct-2026)</t>
         </is>
       </c>
     </row>
@@ -6749,6 +6961,23 @@
       <c r="C9" s="11" t="inlineStr">
         <is>
           <t>Define scenario 6, then add it to the Stage DMS Flow sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>tests/enquiryListReport.spec.ts</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Product-wise Sales Invoice / Booking and the combined summary were removed on 01-Oct while ENQ-08 to 14 stayed marked Pass</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Fixed (08-Oct-2026): rebuilt, with data checks; summary saved to Excel</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stage DMS: enquiry validation tests, clean-up test, steadier TC02
- TC07-TC10: empty enquiry, 5-digit mobile, letters in mobile, field length
  limits; nothing is saved
- TC06: cancel the TC05 receipt; skipped with the reason while the stage user
  has no permission to cancel receipts or bookings
- TC02: retry opening My Enquiries when the DMS's own redirect interrupts it
- Test cases: ENQ-14 passed on an emailed run in Edge; STG-06 to STG-10

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Test Cases/DMS_Automation_Test_Cases.xlsx
+++ b/Test Cases/DMS_Automation_Test_Cases.xlsx
@@ -602,7 +602,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Enquiry List, GSTR and MIS test cases executed on 25-Sep-2026; PDI Vehicle Details and ENQ-16/17 on 28-Sep-2026; PDI master, tracking and email cases (PDI-25 to PDI-32) on 01-Oct-2026 — all against the live DMS (Microsoft Edge and Google Chrome). PDI-29 / PDI-30 are pending the report owner's review of the email. Stage DMS flow (STG-01 to STG-05) on 06-Oct-2026 against the stage DMS (Google Chrome). Enquiry List rebuilt on 08-Oct-2026 (ENQ-05 to ENQ-21, Google Chrome); ENQ-14 is pending an emailed run.</t>
+          <t>Enquiry List, GSTR and MIS test cases executed on 25-Sep-2026; PDI Vehicle Details and ENQ-16/17 on 28-Sep-2026; PDI master, tracking and email cases (PDI-25 to PDI-32) on 01-Oct-2026 — all against the live DMS (Microsoft Edge and Google Chrome). PDI-29 / PDI-30 are pending the report owner's review of the email. Stage DMS flow (STG-01 to STG-05) on 06-Oct-2026 against the stage DMS (Google Chrome). Enquiry List rebuilt on 08-Oct-2026 (ENQ-05 to ENQ-21, Google Chrome); ENQ-14 passed on an emailed run in Microsoft Edge. Stage DMS validation STG-07 to STG-10 passed on 08-Oct-2026; STG-06 (clean-up) is skipped until the stage user can cancel receipts and bookings.</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
         <v>2</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
@@ -788,19 +788,19 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
@@ -816,19 +816,19 @@
       </c>
       <c r="B10" s="6" t="inlineStr"/>
       <c r="C10" s="6" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="H10" s="6" t="inlineStr"/>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="K10" s="11" t="inlineStr">
         <is>
-          <t>All three reports over the limit: Enquiry 31,972, Invoice 5,112, Booking 7,649 rows</t>
+          <t>All three reports over the limit: Enquiry 31,972, Invoice 5,112, Booking 7,649 rows. Also passed in Microsoft Edge on 08-Oct-2026</t>
         </is>
       </c>
     </row>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="J17" s="13" t="inlineStr">
         <is>
-          <t>Pending (08-Oct-2026)</t>
+          <t>Pass (08-Oct-2026)</t>
         </is>
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>Rebuilt 08-Oct. The verification runs had email switched off; confirm on the next CI or local run</t>
+          <t>Rebuilt 08-Oct. Emailed to the GMAIL_TO address with 1 report pasted in the body (run in Microsoft Edge)</t>
         </is>
       </c>
     </row>
@@ -6387,7 +6387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6531,7 +6531,7 @@
       </c>
       <c r="J5" s="13" t="inlineStr">
         <is>
-          <t>Pass (06-Oct-2026)</t>
+          <t>Pass (08-Oct-2026)</t>
         </is>
       </c>
       <c r="K5" s="11" t="inlineStr">
@@ -6594,7 +6594,7 @@
       </c>
       <c r="J6" s="13" t="inlineStr">
         <is>
-          <t>Pass (06-Oct-2026)</t>
+          <t>Pass (08-Oct-2026)</t>
         </is>
       </c>
       <c r="K6" s="11" t="inlineStr">
@@ -6655,7 +6655,7 @@
       </c>
       <c r="J7" s="13" t="inlineStr">
         <is>
-          <t>Pass (06-Oct-2026)</t>
+          <t>Pass (08-Oct-2026)</t>
         </is>
       </c>
       <c r="K7" s="11" t="inlineStr">
@@ -6716,7 +6716,7 @@
       </c>
       <c r="J8" s="13" t="inlineStr">
         <is>
-          <t>Pass (06-Oct-2026)</t>
+          <t>Pass (08-Oct-2026)</t>
         </is>
       </c>
       <c r="K8" s="11" t="inlineStr">
@@ -6777,12 +6777,292 @@
       </c>
       <c r="J9" s="13" t="inlineStr">
         <is>
-          <t>Pass (06-Oct-2026)</t>
+          <t>Pass (08-Oct-2026)</t>
         </is>
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
           <t>Spec test TC05. 06-Oct run: receipt 37200726Ca00019, balance ₹156,499.45</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>STG-06</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Clean-up</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Cancel the receipt made in STG-05</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>Receipt from STG-05</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>1. Open the receipt page
+2. Click Cancel on the receipt row</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr"/>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>Receipt cancelled; Customer Center balance back to the full amount</t>
+        </is>
+      </c>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>Skipped (08-Oct-2026)</t>
+        </is>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>Spec test TC06. The stage River User gets "You do not have permission" on ReceiptCancel.aspx and on Cancel booking. Each run leaves an enquiry, booking and ₹5,000 receipt on stage until a DMS admin grants receipt and booking cancel rights</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>STG-07</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Enquiry with nothing filled in</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>Logged in</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>1. My Enquiries &gt; New
+2. Save without filling anything</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr"/>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>Alert "Please select Source of enquiry"; no enquiry opened</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>Pass (08-Oct-2026)</t>
+        </is>
+      </c>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>Spec test TC07</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>STG-08</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Enquiry with a 5-digit mobile number</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>Logged in</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>1. Fill every mandatory field, mobile 98765
+2. Save</t>
+        </is>
+      </c>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>Mobile 98765</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>Alert "Please check the form once before save. Some of the validations are not matching."; save never sent to the server</t>
+        </is>
+      </c>
+      <c r="J12" s="13" t="inlineStr">
+        <is>
+          <t>Pass (08-Oct-2026)</t>
+        </is>
+      </c>
+      <c r="K12" s="11" t="inlineStr">
+        <is>
+          <t>Spec test TC08</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>STG-09</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Letters typed into the mobile number</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>Logged in</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>Type abcdefghij into Mobile</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr">
+        <is>
+          <t>abcdefghij</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>Field stays empty</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr">
+        <is>
+          <t>Pass (08-Oct-2026)</t>
+        </is>
+      </c>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>Spec test TC09</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>STG-10</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Mobile number and Pin Code length limits</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>Logged in</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>Type 12 digits into Mobile and 7 into Pin Code</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t>987654321012 / 5600011</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>Mobile keeps 11 digits (maxlength 11), Pin Code 6 (maxlength 6)</t>
+        </is>
+      </c>
+      <c r="J14" s="13" t="inlineStr">
+        <is>
+          <t>Pass (08-Oct-2026)</t>
+        </is>
+      </c>
+      <c r="K14" s="11" t="inlineStr">
+        <is>
+          <t>Spec test TC10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
GSTR: stop at once when ProductWise Sales Details is missing from the menu
The DMS removed MIS > Accounts Reports > GSTR Reports > ProductWise Sales
Details (MIS check 08-Oct: 10 Accounts reports left the menu since 29-Sep).
The spec now fails on the first dealer with a message listing what the page
shows, instead of 14 timeouts. GSTR-04 marked Blocked in the test cases.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Test Cases/DMS_Automation_Test_Cases.xlsx
+++ b/Test Cases/DMS_Automation_Test_Cases.xlsx
@@ -602,7 +602,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Enquiry List, GSTR and MIS test cases executed on 25-Sep-2026; PDI Vehicle Details and ENQ-16/17 on 28-Sep-2026; PDI master, tracking and email cases (PDI-25 to PDI-32) on 01-Oct-2026 — all against the live DMS (Microsoft Edge and Google Chrome). PDI-29 / PDI-30 are pending the report owner's review of the email. Stage DMS flow (STG-01 to STG-05) on 06-Oct-2026 against the stage DMS (Google Chrome). Enquiry List rebuilt on 08-Oct-2026 (ENQ-05 to ENQ-21, Google Chrome); ENQ-14 passed on an emailed run in Microsoft Edge. Stage DMS validation STG-07 to STG-10 passed on 08-Oct-2026; STG-06 (clean-up) is skipped until the stage user can cancel receipts and bookings.</t>
+          <t>Enquiry List, GSTR and MIS test cases executed on 25-Sep-2026; PDI Vehicle Details and ENQ-16/17 on 28-Sep-2026; PDI master, tracking and email cases (PDI-25 to PDI-32) on 01-Oct-2026 — all against the live DMS (Microsoft Edge and Google Chrome). PDI-29 / PDI-30 are pending the report owner's review of the email. Stage DMS flow (STG-01 to STG-05) on 06-Oct-2026 against the stage DMS (Google Chrome). Enquiry List rebuilt on 08-Oct-2026 (ENQ-05 to ENQ-21, Google Chrome); ENQ-14 passed on an emailed run in Microsoft Edge. Stage DMS validation STG-07 to STG-10 passed on 08-Oct-2026; STG-06 (clean-up) is skipped until the stage user can cancel receipts and bookings. GSTR Report is blocked from 08-Oct-2026: the DMS removed ProductWise Sales Details from the GSTR Reports menu.</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
         <v>5</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
@@ -828,7 +828,7 @@
         <v>17</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H10" s="6" t="inlineStr"/>
     </row>
@@ -2352,10 +2352,14 @@
       </c>
       <c r="J8" s="13" t="inlineStr">
         <is>
-          <t>Pass (25-Sep-2026)</t>
-        </is>
-      </c>
-      <c r="K8" s="11" t="inlineStr"/>
+          <t>Blocked (08-Oct-2026)</t>
+        </is>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>ProductWise Sales Details is no longer in MIS &gt; Accounts Reports &gt; GSTR Reports for any of the 7 dealers (MIS check 08-Oct lists it as removed). The spec now stops at once with that message. Waiting for the DMS team to restore it or name the replacement</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
@@ -7083,7 +7087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -7261,6 +7265,23 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>tests/GSTR Report.spec.ts</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>DMS removed MIS &gt; Accounts Reports &gt; GSTR Reports &gt; ProductWise Sales Details (found 08-Oct-2026). 10 Accounts reports left the menu since 29-Sep</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Ask the DMS team where the report went; then point the spec at it. Until then the spec fails at once with a clear message</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" copies="1"/>

</xml_diff>